<commit_message>
docs: record the branch-switch incident (E24, Q38, Q39) in the xlsx and research log
在 agenduck 自己的主目录工作区里单击分支，面板没确认就把仓库切到旧分支，正在跑的 AgentDeck 热更新成旧代码。已切回 main 并重启。

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/status/AgentDeck-端到端用例与问题清单-2026-10-24.xlsx
+++ b/docs/status/AgentDeck-端到端用例与问题清单-2026-10-24.xlsx
@@ -13,8 +13,8 @@
     <sheet name="汇总" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'端到端用例'!$A$1:$L$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'问题清单'!$A$1:$K$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'端到端用例'!$A$1:$L$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'问题清单'!$A$1:$K$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -678,7 +678,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24，基于 main 5dfcbe3。证据来自各包测试、apps/desktop/ASSEMBLY_NOTES.md、2026-10-23 的组装和两次启动截图。</t>
+          <t>2026-10-24，基于 main 01947e0（下午补了 E24、Q38、Q39）。证据来自各包测试、apps/desktop/ASSEMBLY_NOTES.md、2026-10-23 的组装和两次启动截图。</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -999,1158 +999,1163 @@
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
+          <t>E24</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>⚠ 当前有问题</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="inlineStr">
+        <is>
+          <t>在面板里给“主目录工作区”切换分支</t>
+        </is>
+      </c>
+      <c r="E2" s="18" t="inlineStr">
+        <is>
+          <t>主目录工作区的框里开着终端（空闲也算）；项目是一个普通测试仓库，不要用 agenduck 本身</t>
+        </is>
+      </c>
+      <c r="F2" s="18" t="inlineStr">
+        <is>
+          <t>1. 聚焦框里的终端
+2. 面板里单击分支按钮
+3. 单击另一个分支</t>
+        </is>
+      </c>
+      <c r="G2" s="18" t="inlineStr">
+        <is>
+          <t>UI：只要这个目录里有终端开着（不管 Running 还是 Idle），先弹确认，写明哪些终端在这个目录里、它们看到的文件会变；确认后才切换，框标题更新为新分支。
+后台：确认后才执行 git switch；切换后 workspace-service 更新记录并发 workspace.changed。</t>
+        </is>
+      </c>
+      <c r="H2" s="18" t="inlineStr">
+        <is>
+          <t>不会因为点错一下就把正在用的目录切到别的分支</t>
+        </is>
+      </c>
+      <c r="I2" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 实际发生：在 agenduck 自己的主目录工作区里单击分支，没有任何确认就把仓库从 main 切到了一个遗留分支（终端都是 Idle，面板只在有改动或有 Running 的 agent 时才确认）；而 AgentDeck 正是从这个目录运行的，开发服务器立刻加载了旧代码，界面变成早期自检页并报错（Q38、Q39）</t>
+        </is>
+      </c>
+      <c r="J2" s="20" t="inlineStr">
+        <is>
+          <t>Q38 Q39 Q31</t>
+        </is>
+      </c>
+      <c r="K2" s="21" t="n"/>
+      <c r="L2" s="22" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
           <t>E04</t>
         </is>
       </c>
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C2" s="17" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D2" s="18" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>agent 停下来请求批准时，用户一眼看出是谁在等</t>
         </is>
       </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>框里有一个已信任文件夹的 claude；应用分别在前台、后台各试一次</t>
         </is>
       </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="F3" s="18" t="inlineStr">
         <is>
           <t>1. 让 claude 执行一个需要批准的命令（例如 “run ls in a new shell”）
 2. 不点任何东西，观察 2 秒
 3. 切到别的应用，再触发一次</t>
         </is>
       </c>
-      <c r="G2" s="18" t="inlineStr">
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>UI：2 秒内窗口出现橙色边框，标题栏状态 Needs approval，框标题和顶栏显示 “1 waiting”，程序坞角标 1；应用在后台时弹系统通知 “claude in … needs approval”。
 后台：claude 的 PermissionRequest 钩子经 agentdeck-notify 送到钩子 socket，状态机进入 needs-approval 并广播 status.changed。</t>
         </is>
       </c>
-      <c r="H2" s="18" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>不用盯着每个终端，也知道哪个 agent 在等你</t>
         </is>
       </c>
-      <c r="I2" s="19" t="inlineStr">
+      <c r="I3" s="19" t="inlineStr">
         <is>
           <t>claude 还停在“信任这个文件夹”提示时，状态显示 Idle，不变橙（Q06）；真 claude 的批准请求从没端到端跑过（Q01）；系统通知没真弹过（Q14）</t>
         </is>
       </c>
-      <c r="J2" s="20" t="inlineStr">
+      <c r="J3" s="20" t="inlineStr">
         <is>
           <t>Q01 Q06 Q14</t>
         </is>
       </c>
-      <c r="K2" s="21" t="n"/>
-      <c r="L2" s="22" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="K3" s="21" t="n"/>
+      <c r="L3" s="22" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>E05</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D3" s="18" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>跳到在等你的窗口，直接批准，agent 继续干活</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>E04 的状态：有一个 claude 在 Needs approval</t>
         </is>
       </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>1. 按 ⌘J
 2. 在终端里按 claude 的“允许一次”键
 3. 观察状态</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>UI：白板平移到那个窗口并聚焦，橙色边框消失（状态点仍橙）；批准后状态变 Running，“1 waiting” 消失。
 后台：输入经 tmux-host 送进 claude；PostToolUse / 新输出让状态机回到 running。</t>
         </is>
       </c>
-      <c r="H3" s="18" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>从发现到批准一气呵成，不用找窗口</t>
         </is>
       </c>
-      <c r="I3" s="19" t="inlineStr">
+      <c r="I4" s="19" t="inlineStr">
         <is>
           <t>需求写的是“直接按 y”，但 claude 实测“允许一次”是 1 或回车（线 1 核对），y 不确定能用，需要定需求（Q12）；批准后回到运行中没测过（Q01）</t>
         </is>
       </c>
-      <c r="J3" s="20" t="inlineStr">
+      <c r="J4" s="20" t="inlineStr">
         <is>
           <t>Q01 Q12</t>
         </is>
       </c>
-      <c r="K3" s="21" t="n"/>
-      <c r="L3" s="22" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="K4" s="21" t="n"/>
+      <c r="L4" s="22" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>E03</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>同一个仓库开两个工作区，两个 claude 并行改代码互不影响</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>已有项目，已建好 feat/oauth 工作区（E02）</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>1. 再建一个 fix/rate-limit 工作区
 2. 两个框里各新开一个 claude，紧接着连续开
 3. 各让它改一个不同的文件</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G5" s="18" t="inlineStr">
         <is>
           <t>UI：两个框各自显示自己的分支，两个 claude 都正常启动；右侧面板随聚焦切换，只显示各自 worktree 的改动。
 后台：两个 worktree 各有自己的 HEAD 和暂存区；两个 tmux 会话的工作目录分别是两个 worktree。</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="H5" s="18" t="inlineStr">
         <is>
           <t>多个 agent 在同一仓库的不同分支上同时工作，改动不串</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="I5" s="19" t="inlineStr">
         <is>
           <t>连着新建两个终端时，第二个可能误显示 “Previous session ended”（Q07）；两个真 claude 并行从没试过（Q03）</t>
         </is>
       </c>
-      <c r="J4" s="20" t="inlineStr">
+      <c r="J5" s="20" t="inlineStr">
         <is>
           <t>Q03 Q07</t>
         </is>
       </c>
-      <c r="K4" s="21" t="n"/>
-      <c r="L4" s="22" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="K5" s="21" t="n"/>
+      <c r="L5" s="22" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>E10</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>退出应用再打开，所有东西都还在</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>白板上有框和至少两个终端，其中一个在跑</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>1. ⌘Q 退出
 2. 再打开（pnpm dev）</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="G6" s="18" t="inlineStr">
         <is>
           <t>UI：框和窗口的位置、大小不变；终端接回，历史输出都在；状态和计时正确。
 后台：tmux 里的会话在应用退出期间一直在跑；重开时按保存的 terminalId 接回，状态机重新登记这些终端。</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr">
+      <c r="H6" s="18" t="inlineStr">
         <is>
           <t>关应用不打断 agent 的工作</t>
         </is>
       </c>
-      <c r="I5" s="19" t="inlineStr">
+      <c r="I6" s="19" t="inlineStr">
         <is>
           <t>接回后状态都显示 “Idle · now”，开始时间没接上（Q08）；强杀进程（不是 ⌘Q）后恢复没测过（Q27）。位置和输出 2026-10-23 已验证</t>
         </is>
       </c>
-      <c r="J5" s="20" t="inlineStr">
+      <c r="J6" s="20" t="inlineStr">
         <is>
           <t>Q08 Q27</t>
         </is>
       </c>
-      <c r="K5" s="21" t="n"/>
-      <c r="L5" s="22" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="K6" s="21" t="n"/>
+      <c r="L6" s="22" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>E02</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>基于 main 新建一个分支工作区，开箱即用</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>已添加项目（E01）；项目里有 .env；设置了初始化命令（例如 pnpm install）</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>1. 右键 › New workspace…
 2. 选 New worktree、New branch，名字 feat/oauth，from main
 3. Create</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="G7" s="18" t="inlineStr">
         <is>
           <t>UI：框出现在右键的位置，标题 “项目 · feat/oauth”；框里自动开一个 Shell 运行初始化命令；右侧面板显示 feat/oauth。
 后台：git worktree add 建好目录并新建分支；.env 被复制过去；失败时已建的 worktree 和分支回滚。</t>
         </is>
       </c>
-      <c r="H6" s="18" t="inlineStr">
+      <c r="H7" s="18" t="inlineStr">
         <is>
           <t>一个新分支的独立工作目录准备好了，agent 可以直接进去干活</t>
         </is>
       </c>
-      <c r="I6" s="19" t="inlineStr">
+      <c r="I7" s="19" t="inlineStr">
         <is>
           <t>从界面新建 worktree 在真窗口里从没走过（Q02）；开发模式下 worktree 放在 .agentdeck-dev 里借用的假主目录下，路径和正式版不同（Q19）</t>
         </is>
       </c>
-      <c r="J6" s="20" t="inlineStr">
+      <c r="J7" s="20" t="inlineStr">
         <is>
           <t>Q02 Q19</t>
         </is>
       </c>
-      <c r="K6" s="21" t="n"/>
-      <c r="L6" s="22" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="K7" s="21" t="n"/>
+      <c r="L7" s="22" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>E15</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>修改项目设置：基础分支、复制的文件、初始化命令</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>已添加项目</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F8" s="18" t="inlineStr">
         <is>
           <t>1. 顶栏 Projects ▾ › Manage projects…（或 Settings › Projects）
 2. 改基础分支和初始化命令
 3. 新建一个工作区验证</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
+      <c r="G8" s="18" t="inlineStr">
         <is>
           <t>UI：有项目设置页，能看到并修改名称、路径、基础分支、worktree 位置、复制的文件、初始化命令。
 后台：设置写进 store，新建工作区时生效。</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="H8" s="18" t="inlineStr">
         <is>
           <t>每个项目按自己的习惯建工作区</t>
         </is>
       </c>
-      <c r="I7" s="19" t="inlineStr">
+      <c r="I8" s="19" t="inlineStr">
         <is>
           <t>没有 Settings 界面：点 Settings 只是用系统程序打开 settings.json，Settings › Projects 不存在（Q13）</t>
         </is>
       </c>
-      <c r="J7" s="20" t="inlineStr">
+      <c r="J8" s="20" t="inlineStr">
         <is>
           <t>Q13</t>
         </is>
       </c>
-      <c r="K7" s="21" t="n"/>
-      <c r="L7" s="22" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="K8" s="21" t="n"/>
+      <c r="L8" s="22" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>E16</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>刚打开应用，右侧面板给出有用的信息</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>白板上有一个工作区框，还没有聚焦任何窗口</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
         <is>
           <t>1. 打开应用，不点任何东西
 2. 单击框里的一个终端</t>
         </is>
       </c>
-      <c r="G8" s="18" t="inlineStr">
+      <c r="G9" s="18" t="inlineStr">
         <is>
           <t>UI：没聚焦时提示怎么开始（例如 “Select a window to see its changes”）；聚焦后显示那个工作区的 git 状态。
 后台：面板只在聚焦变化时刷新一次。</t>
         </is>
       </c>
-      <c r="H8" s="18" t="inlineStr">
+      <c r="H9" s="18" t="inlineStr">
         <is>
           <t>面板不说让人困惑的话</t>
         </is>
       </c>
-      <c r="I8" s="19" t="inlineStr">
+      <c r="I9" s="19" t="inlineStr">
         <is>
           <t>没聚焦任何窗口时也显示 “This window isn’t in a workspace.”（Q22，见重开截图）</t>
         </is>
       </c>
-      <c r="J8" s="20" t="inlineStr">
+      <c r="J9" s="20" t="inlineStr">
         <is>
           <t>Q22</t>
         </is>
       </c>
-      <c r="K8" s="21" t="n"/>
-      <c r="L8" s="22" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="K9" s="21" t="n"/>
+      <c r="L9" s="22" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>E17</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>右键新建终端，菜单只列出能用的 agent</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>本机装了 claude 和 codex</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F10" s="18" t="inlineStr">
         <is>
           <t>1. 在白板空白处右键 › New terminal ▸</t>
         </is>
       </c>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="G10" s="18" t="inlineStr">
         <is>
           <t>UI：列出 Claude、Codex、Shell，用适配器的名字显示；没装的不出现；选中后在点击的位置开终端。
 后台：agents.list() 返回已安装的 agent。</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr">
+      <c r="H10" s="18" t="inlineStr">
         <is>
           <t>菜单里每一项都能用</t>
         </is>
       </c>
-      <c r="I9" s="19" t="inlineStr">
+      <c r="I10" s="19" t="inlineStr">
         <is>
           <t>白板按 agent id 而不是名字显示，并且会列出用不了的 custom；应用里先把 custom 藏掉了，白板包本身没改（Q21）</t>
         </is>
       </c>
-      <c r="J9" s="20" t="inlineStr">
+      <c r="J10" s="20" t="inlineStr">
         <is>
           <t>Q21</t>
         </is>
       </c>
-      <c r="K9" s="21" t="n"/>
-      <c r="L9" s="22" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="K10" s="21" t="n"/>
+      <c r="L10" s="22" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>E01</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C10" s="25" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>未验证</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>第一次打开应用，添加一个项目</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E11" s="18" t="inlineStr">
         <is>
           <t>干净的数据目录（删掉 .agentdeck-dev 或设 AGENTDECK_DATA_DIR 到新目录）；有一个本地 git 仓库</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F11" s="18" t="inlineStr">
         <is>
           <t>1. 在白板空白处右键 › Add project…
 2. 在系统的选文件夹窗口里选仓库（试一次选它的子文件夹）</t>
         </is>
       </c>
-      <c r="G10" s="18" t="inlineStr">
+      <c r="G11" s="18" t="inlineStr">
         <is>
           <t>UI：系统选文件夹窗口出现；选完直接进入 New workspace 对话框，项目已选好；选子文件夹时提示用了仓库根目录。
 后台：projects 表多一条；基础分支自动识别为远端默认分支或 main。</t>
         </is>
       </c>
-      <c r="H10" s="18" t="inlineStr">
+      <c r="H11" s="18" t="inlineStr">
         <is>
           <t>加项目一步到位，直接进入建工作区</t>
         </is>
       </c>
-      <c r="I10" s="18" t="inlineStr">
+      <c r="I11" s="18" t="inlineStr">
         <is>
           <t>流程有单测；组装时用的是演示模式自动加项目，真窗口里没点过</t>
         </is>
       </c>
-      <c r="J10" s="20" t="inlineStr">
+      <c r="J11" s="20" t="inlineStr">
         <is>
           <t>Q02</t>
         </is>
       </c>
-      <c r="K10" s="21" t="n"/>
-      <c r="L10" s="22" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="K11" s="21" t="n"/>
+      <c r="L11" s="22" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>E06</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D11" s="18" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>在框里跑 dev server，点链接就在白板上看效果</t>
         </is>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>框里有一个 Shell 终端；项目能跑 pnpm dev（或用 python3 -m http.server 8765 代替）</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F12" s="18" t="inlineStr">
         <is>
           <t>1. 在终端里运行 dev server
 2. 单击输出里的 localhost 地址
 3. 再单击一次同一个地址</t>
         </is>
       </c>
-      <c r="G11" s="18" t="inlineStr">
+      <c r="G12" s="18" t="inlineStr">
         <is>
           <t>UI：网页窗口出现在终端右边、同一个框里，页面正常显示；第二次单击聚焦并刷新已开的窗口，不新开。
 后台：port-watch 从输出里识别出地址；主进程把这个来源加入响应头改写名单。</t>
         </is>
       </c>
-      <c r="H11" s="18" t="inlineStr">
+      <c r="H12" s="18" t="inlineStr">
         <is>
           <t>写代码和看效果在同一个框里</t>
         </is>
       </c>
-      <c r="I11" s="18" t="inlineStr">
+      <c r="I12" s="18" t="inlineStr">
         <is>
           <t>组装时用 python http.server 点开过网页窗口；真 pnpm dev 和“第二次点击复用”没在真窗口里试</t>
         </is>
       </c>
-      <c r="J11" s="20" t="inlineStr"/>
-      <c r="K11" s="21" t="n"/>
-      <c r="L11" s="22" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="J12" s="20" t="inlineStr"/>
+      <c r="K12" s="21" t="n"/>
+      <c r="L12" s="22" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>E07</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C12" s="26" t="inlineStr">
+      <c r="C13" s="26" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D13" s="18" t="inlineStr">
         <is>
           <t>在右侧面板里提交 agent 改的代码</t>
         </is>
       </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="E13" s="18" t="inlineStr">
         <is>
           <t>某个工作区里有几个改动的文件；用一个测试分支，不要在 main 上提交</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F13" s="18" t="inlineStr">
         <is>
           <t>1. 聚焦那个工作区里的终端
 2. 悬停文件单击 + 暂存两个
 3. 写提交信息，按 ⌘↩</t>
         </is>
       </c>
-      <c r="G12" s="18" t="inlineStr">
+      <c r="G13" s="18" t="inlineStr">
         <is>
           <t>UI：面板显示这个分支的更改，按文件夹树形排列；暂存后进 Staged Changes；提交后列表清空一部分，提交记录顶部出现这一条。
 后台：git add / git commit 在这个 worktree 里执行；提交后面板再刷新一次 status。</t>
         </is>
       </c>
-      <c r="H12" s="18" t="inlineStr">
+      <c r="H13" s="18" t="inlineStr">
         <is>
           <t>不离开白板完成提交</t>
         </is>
       </c>
-      <c r="I12" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>暂存和取消暂存在真窗口里试过；真的提交没做（为了不改 main）</t>
         </is>
       </c>
-      <c r="J12" s="20" t="inlineStr"/>
-      <c r="K12" s="21" t="n"/>
-      <c r="L12" s="22" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="J13" s="20" t="inlineStr"/>
+      <c r="K13" s="21" t="n"/>
+      <c r="L13" s="22" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>E08</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C13" s="25" t="inlineStr">
+      <c r="C14" s="25" t="inlineStr">
         <is>
           <t>未验证</t>
         </is>
       </c>
-      <c r="D13" s="18" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>想切到已被别的工作区占用的分支时，直接跳过去</t>
         </is>
       </c>
-      <c r="E13" s="18" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>同一仓库有 feat/oauth 和 fix/rate-limit 两个工作区（E03）</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="F14" s="18" t="inlineStr">
         <is>
           <t>1. 聚焦 feat/oauth 里的终端
 2. 面板里单击分支按钮
 3. 单击灰显的 fix/rate-limit</t>
         </is>
       </c>
-      <c r="G13" s="18" t="inlineStr">
+      <c r="G14" s="18" t="inlineStr">
         <is>
           <t>UI：fix/rate-limit 灰显并写着 “in fix/rate-limit”；单击后白板平移到那个框并聚焦。
 后台：分支列表来自 git worktree list；不执行任何 git 操作。</t>
         </is>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H14" s="18" t="inlineStr">
         <is>
           <t>不会因为分支被占用而切换失败</t>
         </is>
       </c>
-      <c r="I13" s="18" t="inlineStr">
+      <c r="I14" s="18" t="inlineStr">
         <is>
           <t>面板有单测；需要第二个 worktree，组装时没试</t>
         </is>
       </c>
-      <c r="J13" s="20" t="inlineStr">
+      <c r="J14" s="20" t="inlineStr">
         <is>
           <t>Q25</t>
         </is>
       </c>
-      <c r="K13" s="21" t="n"/>
-      <c r="L13" s="22" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="K14" s="21" t="n"/>
+      <c r="L14" s="22" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>E09</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr">
+      <c r="C15" s="26" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>把终端拉小成摘要卡，腾出地方</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E15" s="18" t="inlineStr">
         <is>
           <t>框里有两个在跑的终端</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F15" s="18" t="inlineStr">
         <is>
           <t>1. 把两个终端的右下角往里拉到很小
 2. 单击其中一个摘要卡</t>
         </is>
       </c>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="G15" s="18" t="inlineStr">
         <is>
           <t>UI：小于 320×200 时变成摘要卡，显示最后 3 行和状态，在等你的仍是橙色；单击恢复到拉小之前的大小并聚焦，画面不乱。
 后台：摘要卡用 capture-pane 取最后几行，不 attach；恢复时重新 attach。</t>
         </is>
       </c>
-      <c r="H14" s="18" t="inlineStr">
+      <c r="H15" s="18" t="inlineStr">
         <is>
           <t>一屏放下更多 agent，又不丢信息</t>
         </is>
       </c>
-      <c r="I14" s="18" t="inlineStr">
+      <c r="I15" s="18" t="inlineStr">
         <is>
           <t>白板和终端窗口都有单测；真窗口里没拉过</t>
         </is>
       </c>
-      <c r="J14" s="20" t="inlineStr">
+      <c r="J15" s="20" t="inlineStr">
         <is>
           <t>Q23</t>
         </is>
       </c>
-      <c r="K14" s="21" t="n"/>
-      <c r="L14" s="22" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="K15" s="21" t="n"/>
+      <c r="L15" s="22" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>E11</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C15" s="25" t="inlineStr">
+      <c r="C16" s="25" t="inlineStr">
         <is>
           <t>未验证</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>在系统终端里接上同一个 agent 会话</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>有一个在跑的 claude 终端</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F16" s="18" t="inlineStr">
         <is>
           <t>1. 标题栏右键 › Open in system terminal
 2. 在两边各输入几个字</t>
         </is>
       </c>
-      <c r="G15" s="18" t="inlineStr">
+      <c r="G16" s="18" t="inlineStr">
         <is>
           <t>UI：系统终端打开并显示同一个会话；两边的输入和输出同步。
 后台：执行 tmux -L agentdeck attach-session -t &lt;id&gt;。</t>
         </is>
       </c>
-      <c r="H15" s="18" t="inlineStr">
+      <c r="H16" s="18" t="inlineStr">
         <is>
           <t>需要时可以用自己习惯的终端接着干</t>
         </is>
       </c>
-      <c r="I15" s="18" t="inlineStr">
+      <c r="I16" s="18" t="inlineStr">
         <is>
           <t>命令拼装有单测；组装时没真点（会打开别的应用）</t>
         </is>
       </c>
-      <c r="J15" s="20" t="inlineStr">
+      <c r="J16" s="20" t="inlineStr">
         <is>
           <t>Q15</t>
         </is>
       </c>
-      <c r="K15" s="21" t="n"/>
-      <c r="L15" s="22" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="K16" s="21" t="n"/>
+      <c r="L16" s="22" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>E12</t>
         </is>
       </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C16" s="26" t="inlineStr">
+      <c r="C17" s="26" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>删除工作区，连目录一起删</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E17" s="18" t="inlineStr">
         <is>
           <t>一个 worktree 工作区，里面有一个未提交的改动；用测试分支</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>1. 右键框 › Delete workspace…
 2. 选 Also delete the worktree folder
 3. 确认；看到“有未提交的更改”再确认一次</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="G17" s="18" t="inlineStr">
         <is>
           <t>UI：第一次确认后提示有未提交的更改，必须再确认；完成后框从白板消失。
 后台：git worktree remove --force；目录从磁盘消失，分支保留。</t>
         </is>
       </c>
-      <c r="H16" s="18" t="inlineStr">
+      <c r="H17" s="18" t="inlineStr">
         <is>
           <t>清理干净，又不会误删还没提交的工作</t>
         </is>
       </c>
-      <c r="I16" s="18" t="inlineStr">
+      <c r="I17" s="18" t="inlineStr">
         <is>
           <t>服务层有真 git 测试；真窗口里没走过。会删目录，要在测试仓库上试</t>
         </is>
       </c>
-      <c r="J16" s="20" t="inlineStr">
+      <c r="J17" s="20" t="inlineStr">
         <is>
           <t>Q24</t>
         </is>
       </c>
-      <c r="K16" s="21" t="n"/>
-      <c r="L16" s="22" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="K17" s="21" t="n"/>
+      <c r="L17" s="22" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>E13</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B18" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C17" s="26" t="inlineStr">
+      <c r="C18" s="26" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D17" s="18" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>关掉窗口，agent 在后台继续，需要时通知你</t>
         </is>
       </c>
-      <c r="E17" s="18" t="inlineStr">
+      <c r="E18" s="18" t="inlineStr">
         <is>
           <t>有一个在跑的 claude</t>
         </is>
       </c>
-      <c r="F17" s="18" t="inlineStr">
+      <c r="F18" s="18" t="inlineStr">
         <is>
           <t>1. 单击窗口的关闭按钮（不是 ⌘Q）
 2. 等 claude 请求批准
 3. 单击系统通知</t>
         </is>
       </c>
-      <c r="G17" s="18" t="inlineStr">
+      <c r="G18" s="18" t="inlineStr">
         <is>
           <t>UI：窗口消失，应用留在程序坞；有批准请求时弹系统通知、角标变 1；单击通知窗口回来并跳到那个终端。
 后台：界面销毁但主进程和 tmux 连接还在；钩子照常到达。</t>
         </is>
       </c>
-      <c r="H17" s="18" t="inlineStr">
+      <c r="H18" s="18" t="inlineStr">
         <is>
           <t>关窗口不等于停工</t>
         </is>
       </c>
-      <c r="I17" s="18" t="inlineStr">
+      <c r="I18" s="18" t="inlineStr">
         <is>
           <t>关窗口后台继续、点程序坞图标回来在真窗口里试过；点系统通知没试</t>
         </is>
       </c>
-      <c r="J17" s="20" t="inlineStr">
+      <c r="J18" s="20" t="inlineStr">
         <is>
           <t>Q14</t>
         </is>
       </c>
-      <c r="K17" s="21" t="n"/>
-      <c r="L17" s="22" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="K18" s="21" t="n"/>
+      <c r="L18" s="22" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>E18</t>
         </is>
       </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C18" s="26" t="inlineStr">
+      <c r="C19" s="26" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>焦点在网页窗口里时，应用快捷键照样能用</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E19" s="18" t="inlineStr">
         <is>
           <t>白板上有一个网页窗口和一个终端</t>
         </is>
       </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>1. 单击网页内容
 2. 用真键盘按 ⌘J、⌘B、⌘W、⌘0、⌘1
 3. 在网页里按 ⌘R</t>
         </is>
       </c>
-      <c r="G18" s="18" t="inlineStr">
+      <c r="G19" s="18" t="inlineStr">
         <is>
           <t>UI：⌘J / ⌘B / ⌘W / ⌘0 / ⌘1 照常生效；⌘R 只刷新这个网页，不重载整个应用。
 后台：快捷键注册成应用菜单的 accelerator。</t>
         </is>
       </c>
-      <c r="H18" s="18" t="inlineStr">
+      <c r="H19" s="18" t="inlineStr">
         <is>
           <t>不管焦点在哪，快捷键行为一致</t>
         </is>
       </c>
-      <c r="I18" s="18" t="inlineStr">
+      <c r="I19" s="18" t="inlineStr">
         <is>
           <t>只用菜单项触发过 ⌘B、⌘W；真键盘没试</t>
         </is>
       </c>
-      <c r="J18" s="20" t="inlineStr">
+      <c r="J19" s="20" t="inlineStr">
         <is>
           <t>Q16</t>
         </is>
       </c>
-      <c r="K18" s="21" t="n"/>
-      <c r="L18" s="22" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="K19" s="21" t="n"/>
+      <c r="L19" s="22" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>E19</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C19" s="25" t="inlineStr">
+      <c r="C20" s="25" t="inlineStr">
         <is>
           <t>未验证</t>
         </is>
       </c>
-      <c r="D19" s="18" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>没装 tmux 或版本太低时给出明确的指引</t>
         </is>
       </c>
-      <c r="E19" s="18" t="inlineStr">
+      <c r="E20" s="18" t="inlineStr">
         <is>
           <t>临时把 PATH 里的 tmux 去掉，或用一个低于 3.5 的 tmux</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="F20" s="18" t="inlineStr">
         <is>
           <t>1. 启动应用
 2. 按提示安装后点 Retry</t>
         </is>
       </c>
-      <c r="G19" s="18" t="inlineStr">
+      <c r="G20" s="18" t="inlineStr">
         <is>
           <t>UI：显示说明页，写明需要 tmux ≥ 3.5 和 brew install tmux，有 Retry；装好后 Retry 能起来。
 后台：启动时检查 tmux -V；低于 3.5 抛 tmux-unavailable。</t>
         </is>
       </c>
-      <c r="H19" s="18" t="inlineStr">
+      <c r="H20" s="18" t="inlineStr">
         <is>
           <t>第一次用的人知道该做什么</t>
         </is>
       </c>
-      <c r="I19" s="18" t="inlineStr">
+      <c r="I20" s="18" t="inlineStr">
         <is>
           <t>版本检查有单测；说明页在真窗口里没看过</t>
         </is>
       </c>
-      <c r="J19" s="20" t="inlineStr"/>
-      <c r="K19" s="21" t="n"/>
-      <c r="L19" s="22" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="J20" s="20" t="inlineStr"/>
+      <c r="K20" s="21" t="n"/>
+      <c r="L20" s="22" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>E20</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C20" s="25" t="inlineStr">
+      <c r="C21" s="25" t="inlineStr">
         <is>
           <t>未验证</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>从程序坞打开应用，agent 照样能联网、能登录</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E21" s="18" t="inlineStr">
         <is>
           <t>需要打包好的应用（现在还没有打包流程）</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F21" s="18" t="inlineStr">
         <is>
           <t>1. 从程序坞或访达打开 AgentDeck
 2. 新开一个 claude，发一句话</t>
         </is>
       </c>
-      <c r="G20" s="18" t="inlineStr">
+      <c r="G21" s="18" t="inlineStr">
         <is>
           <t>UI：claude 正常回答，不出现 403 或找不到命令。
 后台：启动时读登录 shell 的环境（PATH、代理变量），传给 tmux-host 和适配器。</t>
         </is>
       </c>
-      <c r="H20" s="18" t="inlineStr">
+      <c r="H21" s="18" t="inlineStr">
         <is>
           <t>不管从哪里打开，体验都和终端里一样</t>
         </is>
       </c>
-      <c r="I20" s="18" t="inlineStr">
+      <c r="I21" s="18" t="inlineStr">
         <is>
           <t>只从终端里 pnpm dev 启动过，那时环境本来就是全的；从程序坞启动要等有打包版本（Q11、Q37）</t>
         </is>
       </c>
-      <c r="J20" s="20" t="inlineStr">
+      <c r="J21" s="20" t="inlineStr">
         <is>
           <t>Q11 Q37</t>
         </is>
       </c>
-      <c r="K20" s="21" t="n"/>
-      <c r="L20" s="22" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="K21" s="21" t="n"/>
+      <c r="L21" s="22" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>E21</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C21" s="27" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
         <is>
           <t>已验证</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>右键在白板上开一个终端并使用</t>
         </is>
       </c>
-      <c r="E21" s="18" t="inlineStr">
+      <c r="E22" s="18" t="inlineStr">
         <is>
           <t>应用已打开</t>
         </is>
       </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="F22" s="18" t="inlineStr">
         <is>
           <t>1. 空白处右键 › New terminal ▸ Shell
 2. 输入 git status</t>
         </is>
       </c>
-      <c r="G21" s="18" t="inlineStr">
+      <c r="G22" s="18" t="inlineStr">
         <is>
           <t>UI：在点击的位置出现终端，散放的终端在 ~ 运行；输出正常显示，状态 Running 后变 Idle。
 后台：tmux 里新建会话，窗格带 AGENTDECK_TERM；输出经 MessagePort 直达界面。</t>
         </is>
       </c>
-      <c r="H21" s="18" t="inlineStr">
+      <c r="H22" s="18" t="inlineStr">
         <is>
           <t>白板上直接用真终端</t>
-        </is>
-      </c>
-      <c r="I21" s="18" t="inlineStr">
-        <is>
-          <t>2026-10-23 组装时验证</t>
-        </is>
-      </c>
-      <c r="J21" s="20" t="inlineStr"/>
-      <c r="K21" s="21" t="n"/>
-      <c r="L21" s="22" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>E22</t>
-        </is>
-      </c>
-      <c r="B22" s="23" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C22" s="27" t="inlineStr">
-        <is>
-          <t>已验证</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>关闭运行中的终端会结束进程</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>有一个在跑的终端</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>1. 单击标题栏的关闭
-2. 在确认框里选结束并关闭</t>
-        </is>
-      </c>
-      <c r="G22" s="18" t="inlineStr">
-        <is>
-          <t>UI：先弹确认；确认后窗口消失。
-后台：tmux 会话被结束。</t>
-        </is>
-      </c>
-      <c r="H22" s="18" t="inlineStr">
-        <is>
-          <t>关窗口不会留下看不见的进程</t>
         </is>
       </c>
       <c r="I22" s="18" t="inlineStr">
@@ -2165,7 +2170,7 @@
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>E23</t>
+          <t>E22</t>
         </is>
       </c>
       <c r="B23" s="23" t="inlineStr">
@@ -2180,34 +2185,34 @@
       </c>
       <c r="D23" s="18" t="inlineStr">
         <is>
-          <t>在面板里暂存再取消暂存一个文件</t>
+          <t>关闭运行中的终端会结束进程</t>
         </is>
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>工作区里有一个改动</t>
+          <t>有一个在跑的终端</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>1. 单击文件旁的 +
-2. 再单击 −</t>
+          <t>1. 单击标题栏的关闭
+2. 在确认框里选结束并关闭</t>
         </is>
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
-          <t>UI：文件在 Changes 和 Staged Changes 之间移动。
-后台：git add / git restore --staged；git status 和界面一致。</t>
+          <t>UI：先弹确认；确认后窗口消失。
+后台：tmux 会话被结束。</t>
         </is>
       </c>
       <c r="H23" s="18" t="inlineStr">
         <is>
-          <t>暂存操作和命令行一致</t>
+          <t>关窗口不会留下看不见的进程</t>
         </is>
       </c>
       <c r="I23" s="18" t="inlineStr">
         <is>
-          <t>2026-10-23 组装时验证（两次都对照了 git status）</t>
+          <t>2026-10-23 组装时验证</t>
         </is>
       </c>
       <c r="J23" s="20" t="inlineStr"/>
@@ -2217,62 +2222,114 @@
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>已验证</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>在面板里暂存再取消暂存一个文件</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>工作区里有一个改动</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>1. 单击文件旁的 +
+2. 再单击 −</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>UI：文件在 Changes 和 Staged Changes 之间移动。
+后台：git add / git restore --staged；git status 和界面一致。</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>暂存操作和命令行一致</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-23 组装时验证（两次都对照了 git status）</t>
+        </is>
+      </c>
+      <c r="J24" s="20" t="inlineStr"/>
+      <c r="K24" s="21" t="n"/>
+      <c r="L24" s="22" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
           <t>E14</t>
         </is>
       </c>
-      <c r="B24" s="24" t="inlineStr">
+      <c r="B25" s="24" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C24" s="28" t="inlineStr">
+      <c r="C25" s="28" t="inlineStr">
         <is>
           <t>未实现</t>
         </is>
       </c>
-      <c r="D24" s="18" t="inlineStr">
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>重启电脑后恢复上次的工作区和 agent 对话</t>
         </is>
       </c>
-      <c r="E24" s="18" t="inlineStr">
+      <c r="E25" s="18" t="inlineStr">
         <is>
           <t>电脑重启过（或 tmux kill-server 模拟）</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr">
+      <c r="F25" s="18" t="inlineStr">
         <is>
           <t>1. 打开应用
 2. 在 “Restore your last session?” 里选 Restore all</t>
         </is>
       </c>
-      <c r="G24" s="18" t="inlineStr">
+      <c r="G25" s="18" t="inlineStr">
         <is>
           <t>UI：弹出恢复提示；恢复后工作区和窗口在原位，claude 接回原来的对话，Shell 在原目录打开并填好命令。
 后台：按记录的会话 id 运行 claude --resume &lt;id&gt;、codex resume &lt;id&gt;。</t>
         </is>
       </c>
-      <c r="H24" s="18" t="inlineStr">
+      <c r="H25" s="18" t="inlineStr">
         <is>
           <t>重启不丢上下文</t>
         </is>
       </c>
-      <c r="I24" s="18" t="inlineStr">
+      <c r="I25" s="18" t="inlineStr">
         <is>
           <t>属于 MVP 完整版（M4 · X6），还没做</t>
         </is>
       </c>
-      <c r="J24" s="20" t="inlineStr">
+      <c r="J25" s="20" t="inlineStr">
         <is>
           <t>Q36</t>
         </is>
       </c>
-      <c r="K24" s="21" t="n"/>
-      <c r="L24" s="22" t="n"/>
+      <c r="K25" s="21" t="n"/>
+      <c r="L25" s="22" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L24"/>
-  <conditionalFormatting sqref="K2:K24">
+  <autoFilter ref="A1:L25"/>
+  <conditionalFormatting sqref="K2:K25">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$K2="不通过"</formula>
     </cfRule>
@@ -2281,7 +2338,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"通过,不通过,阻塞,跳过"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2295,7 +2352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2632,12 +2689,12 @@
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Q06</t>
-        </is>
-      </c>
-      <c r="B7" s="23" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Q38</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -2647,32 +2704,32 @@
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>agent-adapters</t>
+          <t>源代码管理面板 · 白板</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>claude 停在“信任这个文件夹”提示时，状态显示 Idle，应该算在等你</t>
+          <t>在面板里单击分支会立刻切换，不确认：只有在有未提交改动或有 Running 的 agent 时才弹框；框里的终端是 Idle 时直接切。空闲的 agent 和 Shell 也在这个目录里，切分支会改掉它们眼前的文件</t>
         </is>
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>打开一个没信任过的目录里的 claude</t>
+          <t>主目录工作区里开一个 Idle 的终端，在面板里单击另一个分支</t>
         </is>
       </c>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>用户以为 claude 在空闲，其实它卡着等你</t>
+          <t>误点一下就切走正在用的目录；2026-10-24 验收时实际发生</t>
         </is>
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>状态机把启动后迟迟没有 SessionStart、且屏幕停住的情况算 needs-reply，或识别信任提示</t>
+          <t>只要这个目录里有任何终端开着就先确认（白板把框里所有活着的终端传给面板，不只 Running 的）；确认框写清会受影响的终端</t>
         </is>
       </c>
       <c r="I7" s="20" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E24</t>
         </is>
       </c>
       <c r="J7" s="21" t="inlineStr">
@@ -2685,47 +2742,47 @@
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Q07</t>
-        </is>
-      </c>
-      <c r="B8" s="23" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Q39</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>缺陷</t>
+          <t>开发风险</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>终端窗口</t>
+          <t>apps/desktop · 开发流程</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>连着新建两个终端时，第二个可能误显示 “Previous session ended”（它复用了 500 毫秒内的 terminals.list() 结果）</t>
+          <t>用 AgentDeck 管理 agenduck 仓库自己时，切换主目录的分支会改掉正在运行的 AgentDeck 的源代码，开发服务器热更新成旧代码，界面直接坏掉</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>快速连开两个终端</t>
+          <t>在 agenduck 自己的主目录工作区里切到任何旧分支</t>
         </is>
       </c>
       <c r="G8" s="18" t="inlineStr">
         <is>
-          <t>用户以为终端没起来</t>
+          <t>验收和自举开发时很容易误伤；恢复要手动 git switch main 再重启</t>
         </is>
       </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>新建后强制刷新列表，或按 terminalId 精确查询</t>
+          <t>短期：验收用别的测试仓库，或在独立 worktree 里跑 pnpm dev；长期：应用检测到要切的目录就是自己运行的目录时拒绝并提示</t>
         </is>
       </c>
       <c r="I8" s="20" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E24</t>
         </is>
       </c>
       <c r="J8" s="21" t="inlineStr">
@@ -2738,7 +2795,7 @@
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>Q09</t>
+          <t>Q06</t>
         </is>
       </c>
       <c r="B9" s="23" t="inlineStr">
@@ -2748,35 +2805,39 @@
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>技术债</t>
+          <t>缺陷</t>
         </is>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>tmux-host</t>
+          <t>agent-adapters</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>pty.ts 自己声明了顶层 const require，和 electron-vite 注入的重名，终端进程一启动就崩；组装时在构建配置里绕过</t>
+          <t>claude 停在“信任这个文件夹”提示时，状态显示 Idle，应该算在等你</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>去掉桌面构建配置里的绕过插件后启动</t>
+          <t>打开一个没信任过的目录里的 claude</t>
         </is>
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>换构建工具或打包时会再炸</t>
+          <t>用户以为 claude 在空闲，其实它卡着等你</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>在 tmux-host 里改名，去掉绕过</t>
-        </is>
-      </c>
-      <c r="I9" s="20" t="inlineStr"/>
+          <t>状态机把启动后迟迟没有 SessionStart、且屏幕停住的情况算 needs-reply，或识别信任提示</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
       <c r="J9" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -2787,7 +2848,7 @@
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>Q10</t>
+          <t>Q07</t>
         </is>
       </c>
       <c r="B10" s="23" t="inlineStr">
@@ -2797,35 +2858,39 @@
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>技术债</t>
+          <t>缺陷</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>tmux-host</t>
+          <t>终端窗口</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>打包后默认的 tmux.conf 路径不对，应用现在总是显式传路径</t>
+          <t>连着新建两个终端时，第二个可能误显示 “Previous session ended”（它复用了 500 毫秒内的 terminals.list() 结果）</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>打包后不传路径启动</t>
+          <t>快速连开两个终端</t>
         </is>
       </c>
       <c r="G10" s="18" t="inlineStr">
         <is>
-          <t>打包时容易漏</t>
+          <t>用户以为终端没起来</t>
         </is>
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>默认路径按打包后的资源目录算</t>
-        </is>
-      </c>
-      <c r="I10" s="20" t="inlineStr"/>
+          <t>新建后强制刷新列表，或按 terminalId 精确查询</t>
+        </is>
+      </c>
+      <c r="I10" s="20" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
       <c r="J10" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -2836,7 +2901,7 @@
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q09</t>
         </is>
       </c>
       <c r="B11" s="23" t="inlineStr">
@@ -2846,39 +2911,35 @@
       </c>
       <c r="C11" s="20" t="inlineStr">
         <is>
-          <t>未验证</t>
+          <t>技术债</t>
         </is>
       </c>
       <c r="D11" s="18" t="inlineStr">
         <is>
-          <t>apps/desktop</t>
+          <t>tmux-host</t>
         </is>
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>从程序坞打开时读登录 shell 环境（PATH、代理）没验证过：只从终端 pnpm dev 启动过，那时环境本来就全</t>
+          <t>pty.ts 自己声明了顶层 const require，和 electron-vite 注入的重名，终端进程一启动就崩；组装时在构建配置里绕过</t>
         </is>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>有打包版本后从程序坞打开，开 claude 发一句话</t>
+          <t>去掉桌面构建配置里的绕过插件后启动</t>
         </is>
       </c>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>之前 403 就是缺代理变量导致的</t>
+          <t>换构建工具或打包时会再炸</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>和 Q37 一起做</t>
-        </is>
-      </c>
-      <c r="I11" s="20" t="inlineStr">
-        <is>
-          <t>E20</t>
-        </is>
-      </c>
+          <t>在 tmux-host 里改名，去掉绕过</t>
+        </is>
+      </c>
+      <c r="I11" s="20" t="inlineStr"/>
       <c r="J11" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -2889,7 +2950,7 @@
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="B12" s="23" t="inlineStr">
@@ -2899,39 +2960,35 @@
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>需求不一致</t>
+          <t>技术债</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>需求 · agent-adapters</t>
+          <t>tmux-host</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>验收场景 5 写“直接按 y 批准”，claude 实测“允许一次”是 1 或回车，y 能不能用不确定</t>
+          <t>打包后默认的 tmux.conf 路径不对，应用现在总是显式传路径</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>在 claude 的批准提示里按 y 试一次</t>
+          <t>打包后不传路径启动</t>
         </is>
       </c>
       <c r="G12" s="18" t="inlineStr">
         <is>
-          <t>按错键可能选到别的选项</t>
+          <t>打包时容易漏</t>
         </is>
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>改需求写法为“按 agent 的允许一次键（claude 是 1）”，或实测 y 后定下</t>
-        </is>
-      </c>
-      <c r="I12" s="20" t="inlineStr">
-        <is>
-          <t>E05</t>
-        </is>
-      </c>
+          <t>默认路径按打包后的资源目录算</t>
+        </is>
+      </c>
+      <c r="I12" s="20" t="inlineStr"/>
       <c r="J12" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -2942,7 +2999,7 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>Q11</t>
         </is>
       </c>
       <c r="B13" s="23" t="inlineStr">
@@ -2952,37 +3009,37 @@
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>未验证</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>白板 · apps/desktop</t>
+          <t>apps/desktop</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>没有 Settings 界面：设置存在 settings.json，点 Settings 用系统程序打开它；需求里的 Settings › Projects、Settings › Agents 都没有</t>
+          <t>从程序坞打开时读登录 shell 环境（PATH、代理）没验证过：只从终端 pnpm dev 启动过，那时环境本来就全</t>
         </is>
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>点顶栏 Settings</t>
+          <t>有打包版本后从程序坞打开，开 claude 发一句话</t>
         </is>
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>项目设置、agent 启动参数、破坏性命令名单都只能手改 JSON</t>
+          <t>之前 403 就是缺代理变量导致的</t>
         </is>
       </c>
       <c r="H13" s="18" t="inlineStr">
         <is>
-          <t>先做 Projects 和 Agents 两页</t>
+          <t>和 Q37 一起做</t>
         </is>
       </c>
       <c r="I13" s="20" t="inlineStr">
         <is>
-          <t>E15</t>
+          <t>E20</t>
         </is>
       </c>
       <c r="J13" s="21" t="inlineStr">
@@ -2995,7 +3052,7 @@
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B14" s="23" t="inlineStr">
@@ -3005,37 +3062,37 @@
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>未验证</t>
+          <t>需求不一致</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>apps/desktop</t>
+          <t>需求 · agent-adapters</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>系统通知真弹出、单击后窗口回来并跳到终端，没验证</t>
+          <t>验收场景 5 写“直接按 y 批准”，claude 实测“允许一次”是 1 或回车，y 能不能用不确定</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>按 E13 走一遍</t>
+          <t>在 claude 的批准提示里按 y 试一次</t>
         </is>
       </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
-          <t>后台提醒是“不用盯着”的关键</t>
+          <t>按错键可能选到别的选项</t>
         </is>
       </c>
       <c r="H14" s="18" t="inlineStr">
         <is>
-          <t>手动验收 E13</t>
+          <t>改需求写法为“按 agent 的允许一次键（claude 是 1）”，或实测 y 后定下</t>
         </is>
       </c>
       <c r="I14" s="20" t="inlineStr">
         <is>
-          <t>E04 E13</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="J14" s="21" t="inlineStr">
@@ -3048,7 +3105,7 @@
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>Q13</t>
         </is>
       </c>
       <c r="B15" s="23" t="inlineStr">
@@ -3058,37 +3115,37 @@
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
-          <t>未验证</t>
+          <t>缺失</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>apps/desktop · 白板</t>
+          <t>白板 · apps/desktop</t>
         </is>
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>焦点在网页窗口里时，用真键盘按应用快捷键没验证过（只用菜单项触发过）</t>
+          <t>没有 Settings 界面：设置存在 settings.json，点 Settings 用系统程序打开它；需求里的 Settings › Projects、Settings › Agents 都没有</t>
         </is>
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>按 E18 走一遍</t>
+          <t>点顶栏 Settings</t>
         </is>
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>快捷键失灵会很烦</t>
+          <t>项目设置、agent 启动参数、破坏性命令名单都只能手改 JSON</t>
         </is>
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>手动验收 E18</t>
+          <t>先做 Projects 和 Agents 两页</t>
         </is>
       </c>
       <c r="I15" s="20" t="inlineStr">
         <is>
-          <t>E18</t>
+          <t>E15</t>
         </is>
       </c>
       <c r="J15" s="21" t="inlineStr">
@@ -3101,7 +3158,7 @@
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q14</t>
         </is>
       </c>
       <c r="B16" s="23" t="inlineStr">
@@ -3111,35 +3168,39 @@
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>技术债</t>
+          <t>未验证</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>contracts</t>
+          <t>apps/desktop</t>
         </is>
       </c>
       <c r="E16" s="18" t="inlineStr">
         <is>
-          <t>线 1 的 13 条接口意见没整理成 0.1.4：关闭确认不知道进程在不在跑、⌘K 只发 Ctrl+L 没清历史、拖入文件拿不到路径、没有打开外部链接、没有终端配色 token 等</t>
+          <t>系统通知真弹出、单击后窗口回来并跳到终端，没验证</t>
         </is>
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>看 packages/tmux-host/CONTRACT_NOTES.md</t>
+          <t>按 E13 走一遍</t>
         </is>
       </c>
       <c r="G16" s="18" t="inlineStr">
         <is>
-          <t>这些地方现在是各包自己临时处理</t>
+          <t>后台提醒是“不用盯着”的关键</t>
         </is>
       </c>
       <c r="H16" s="18" t="inlineStr">
         <is>
-          <t>出 contracts 0.1.4 并跟进实现</t>
-        </is>
-      </c>
-      <c r="I16" s="20" t="inlineStr"/>
+          <t>手动验收 E13</t>
+        </is>
+      </c>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>E04 E13</t>
+        </is>
+      </c>
       <c r="J16" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -3150,7 +3211,7 @@
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>Q24</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="B17" s="23" t="inlineStr">
@@ -3165,32 +3226,32 @@
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>白板 · workspace-service</t>
+          <t>apps/desktop · 白板</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>在真窗口里删除工作区并删目录没走过（会真删磁盘目录）</t>
+          <t>焦点在网页窗口里时，用真键盘按应用快捷键没验证过（只用菜单项触发过）</t>
         </is>
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>在测试仓库上按 E12 走一遍</t>
+          <t>按 E18 走一遍</t>
         </is>
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>删除是不可逆操作，必须先验证</t>
+          <t>快捷键失灵会很烦</t>
         </is>
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>手动验收 E12</t>
+          <t>手动验收 E18</t>
         </is>
       </c>
       <c r="I17" s="20" t="inlineStr">
         <is>
-          <t>E12</t>
+          <t>E18</t>
         </is>
       </c>
       <c r="J17" s="21" t="inlineStr">
@@ -3203,49 +3264,45 @@
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>Q08</t>
-        </is>
-      </c>
-      <c r="B18" s="24" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>缺陷</t>
+          <t>技术债</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>agent-adapters · contracts</t>
+          <t>contracts</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
         <is>
-          <t>重开应用后终端状态都显示 “Idle · now”，开始时间没接上</t>
+          <t>线 1 的 13 条接口意见没整理成 0.1.4：关闭确认不知道进程在不在跑、⌘K 只发 Ctrl+L 没清历史、拖入文件拿不到路径、没有打开外部链接、没有终端配色 token 等</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>有终端在跑时 ⌘Q 再打开</t>
+          <t>看 packages/tmux-host/CONTRACT_NOTES.md</t>
         </is>
       </c>
       <c r="G18" s="18" t="inlineStr">
         <is>
-          <t>计时不准，但不影响使用</t>
+          <t>这些地方现在是各包自己临时处理</t>
         </is>
       </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
-          <t>状态机接受恢复时的真实开始时间</t>
-        </is>
-      </c>
-      <c r="I18" s="20" t="inlineStr">
-        <is>
-          <t>E10</t>
-        </is>
-      </c>
+          <t>出 contracts 0.1.4 并跟进实现</t>
+        </is>
+      </c>
+      <c r="I18" s="20" t="inlineStr"/>
       <c r="J18" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -3256,12 +3313,12 @@
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>Q15</t>
-        </is>
-      </c>
-      <c r="B19" s="24" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>Q24</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="C19" s="20" t="inlineStr">
@@ -3271,32 +3328,32 @@
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>终端窗口 · apps/desktop</t>
+          <t>白板 · workspace-service</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
         <is>
-          <t>Open in system terminal 没真点过</t>
+          <t>在真窗口里删除工作区并删目录没走过（会真删磁盘目录）</t>
         </is>
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>按 E11 走一遍</t>
+          <t>在测试仓库上按 E12 走一遍</t>
         </is>
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>辅助功能</t>
+          <t>删除是不可逆操作，必须先验证</t>
         </is>
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>手动验收 E11</t>
+          <t>手动验收 E12</t>
         </is>
       </c>
       <c r="I19" s="20" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E12</t>
         </is>
       </c>
       <c r="J19" s="21" t="inlineStr">
@@ -3309,7 +3366,7 @@
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>Q18</t>
+          <t>Q08</t>
         </is>
       </c>
       <c r="B20" s="24" t="inlineStr">
@@ -3319,35 +3376,39 @@
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>技术债</t>
+          <t>缺陷</t>
         </is>
       </c>
       <c r="D20" s="18" t="inlineStr">
         <is>
-          <t>白板 · 网页窗口 · git · agent</t>
+          <t>agent-adapters · contracts</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
         <is>
-          <t>线 2–5 还没把 contracts 0.1.3 的新字段用进代码：白板仍按 type === "terminal" 写特例、reuseKey 不随白板保存、网页窗口用本地的 reloadToken、远端分支和接回已有 worktree 没实现等</t>
+          <t>重开应用后终端状态都显示 “Idle · now”，开始时间没接上</t>
         </is>
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>看各包 CONTRACT_NOTES.md 开头的“待跟进”</t>
+          <t>有终端在跑时 ⌘Q 再打开</t>
         </is>
       </c>
       <c r="G20" s="18" t="inlineStr">
         <is>
-          <t>加新窗口类型时要改白板</t>
+          <t>计时不准，但不影响使用</t>
         </is>
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>各包跟进一轮</t>
-        </is>
-      </c>
-      <c r="I20" s="20" t="inlineStr"/>
+          <t>状态机接受恢复时的真实开始时间</t>
+        </is>
+      </c>
+      <c r="I20" s="20" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J20" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -3358,7 +3419,7 @@
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Q15</t>
         </is>
       </c>
       <c r="B21" s="24" t="inlineStr">
@@ -3368,37 +3429,37 @@
       </c>
       <c r="C21" s="20" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>未验证</t>
         </is>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>workspace-service</t>
+          <t>终端窗口 · apps/desktop</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
         <is>
-          <t>没有“worktree 放在哪”的选项，开发模式下借用 .agentdeck-dev 里的假主目录</t>
+          <t>Open in system terminal 没真点过</t>
         </is>
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>开发模式下新建 worktree，看它的路径</t>
+          <t>按 E11 走一遍</t>
         </is>
       </c>
       <c r="G21" s="18" t="inlineStr">
         <is>
-          <t>开发和正式版路径不一致</t>
+          <t>辅助功能</t>
         </is>
       </c>
       <c r="H21" s="18" t="inlineStr">
         <is>
-          <t>给 workspace-service 加 worktreeRoot 参数</t>
+          <t>手动验收 E11</t>
         </is>
       </c>
       <c r="I21" s="20" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="J21" s="21" t="inlineStr">
@@ -3411,7 +3472,7 @@
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>Q20</t>
+          <t>Q18</t>
         </is>
       </c>
       <c r="B22" s="24" t="inlineStr">
@@ -3421,32 +3482,32 @@
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>缺陷</t>
+          <t>技术债</t>
         </is>
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>白板</t>
+          <t>白板 · 网页窗口 · git · agent</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
         <is>
-          <t>第二次调用 start() 在白板加载完之前就返回</t>
+          <t>线 2–5 还没把 contracts 0.1.3 的新字段用进代码：白板仍按 type === "terminal" 写特例、reuseKey 不随白板保存、网页窗口用本地的 reloadToken、远端分支和接回已有 worktree 没实现等</t>
         </is>
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>连续调用两次 controller.start()</t>
+          <t>看各包 CONTRACT_NOTES.md 开头的“待跟进”</t>
         </is>
       </c>
       <c r="G22" s="18" t="inlineStr">
         <is>
-          <t>应用里已绕过（先 start 再渲染）</t>
+          <t>加新窗口类型时要改白板</t>
         </is>
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>让 start() 返回同一个 Promise</t>
+          <t>各包跟进一轮</t>
         </is>
       </c>
       <c r="I22" s="20" t="inlineStr"/>
@@ -3460,7 +3521,7 @@
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>Q21</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="B23" s="24" t="inlineStr">
@@ -3470,37 +3531,37 @@
       </c>
       <c r="C23" s="20" t="inlineStr">
         <is>
-          <t>缺陷</t>
+          <t>缺失</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
         <is>
-          <t>白板</t>
+          <t>workspace-service</t>
         </is>
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>新建终端菜单会列出用不了的 custom，并按 agent id 而不是名字显示</t>
+          <t>没有“worktree 放在哪”的选项，开发模式下借用 .agentdeck-dev 里的假主目录</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>右键 › New terminal ▸</t>
+          <t>开发模式下新建 worktree，看它的路径</t>
         </is>
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
-          <t>应用里先藏了 custom</t>
+          <t>开发和正式版路径不一致</t>
         </is>
       </c>
       <c r="H23" s="18" t="inlineStr">
         <is>
-          <t>按 AgentInfo.label 显示，过滤 custom</t>
+          <t>给 workspace-service 加 worktreeRoot 参数</t>
         </is>
       </c>
       <c r="I23" s="20" t="inlineStr">
         <is>
-          <t>E17</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="J23" s="21" t="inlineStr">
@@ -3513,7 +3574,7 @@
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>Q22</t>
+          <t>Q20</t>
         </is>
       </c>
       <c r="B24" s="24" t="inlineStr">
@@ -3528,34 +3589,30 @@
       </c>
       <c r="D24" s="18" t="inlineStr">
         <is>
-          <t>源代码管理面板</t>
+          <t>白板</t>
         </is>
       </c>
       <c r="E24" s="18" t="inlineStr">
         <is>
-          <t>没有聚焦任何窗口时也显示 “This window isn’t in a workspace.”</t>
+          <t>第二次调用 start() 在白板加载完之前就返回</t>
         </is>
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>打开应用不点任何东西</t>
+          <t>连续调用两次 controller.start()</t>
         </is>
       </c>
       <c r="G24" s="18" t="inlineStr">
         <is>
-          <t>文案让人困惑</t>
+          <t>应用里已绕过（先 start 再渲染）</t>
         </is>
       </c>
       <c r="H24" s="18" t="inlineStr">
         <is>
-          <t>区分“没聚焦”和“聚焦的是散放窗口”</t>
-        </is>
-      </c>
-      <c r="I24" s="20" t="inlineStr">
-        <is>
-          <t>E16</t>
-        </is>
-      </c>
+          <t>让 start() 返回同一个 Promise</t>
+        </is>
+      </c>
+      <c r="I24" s="20" t="inlineStr"/>
       <c r="J24" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -3566,7 +3623,7 @@
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>Q23</t>
+          <t>Q21</t>
         </is>
       </c>
       <c r="B25" s="24" t="inlineStr">
@@ -3576,37 +3633,37 @@
       </c>
       <c r="C25" s="20" t="inlineStr">
         <is>
-          <t>未验证</t>
+          <t>缺陷</t>
         </is>
       </c>
       <c r="D25" s="18" t="inlineStr">
         <is>
-          <t>白板 · 终端窗口</t>
+          <t>白板</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">
         <is>
-          <t>在真窗口里拉小成摘要卡、再恢复，画面会不会乱没验证</t>
+          <t>新建终端菜单会列出用不了的 custom，并按 agent id 而不是名字显示</t>
         </is>
       </c>
       <c r="F25" s="18" t="inlineStr">
         <is>
-          <t>按 E09 走一遍</t>
+          <t>右键 › New terminal ▸</t>
         </is>
       </c>
       <c r="G25" s="18" t="inlineStr">
         <is>
-          <t>摘要卡是放下更多窗口的办法</t>
+          <t>应用里先藏了 custom</t>
         </is>
       </c>
       <c r="H25" s="18" t="inlineStr">
         <is>
-          <t>手动验收 E09</t>
+          <t>按 AgentInfo.label 显示，过滤 custom</t>
         </is>
       </c>
       <c r="I25" s="20" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>E17</t>
         </is>
       </c>
       <c r="J25" s="21" t="inlineStr">
@@ -3619,7 +3676,7 @@
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>Q25</t>
+          <t>Q22</t>
         </is>
       </c>
       <c r="B26" s="24" t="inlineStr">
@@ -3629,7 +3686,7 @@
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>未验证</t>
+          <t>缺陷</t>
         </is>
       </c>
       <c r="D26" s="18" t="inlineStr">
@@ -3639,27 +3696,27 @@
       </c>
       <c r="E26" s="18" t="inlineStr">
         <is>
-          <t>单击被别的工作区占用的分支跳到那个框，没在真窗口里试</t>
+          <t>没有聚焦任何窗口时也显示 “This window isn’t in a workspace.”</t>
         </is>
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>按 E08 走一遍</t>
+          <t>打开应用不点任何东西</t>
         </is>
       </c>
       <c r="G26" s="18" t="inlineStr">
         <is>
-          <t>辅助功能</t>
+          <t>文案让人困惑</t>
         </is>
       </c>
       <c r="H26" s="18" t="inlineStr">
         <is>
-          <t>手动验收 E08</t>
+          <t>区分“没聚焦”和“聚焦的是散放窗口”</t>
         </is>
       </c>
       <c r="I26" s="20" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="J26" s="21" t="inlineStr">
@@ -3672,7 +3729,7 @@
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>Q26</t>
+          <t>Q23</t>
         </is>
       </c>
       <c r="B27" s="24" t="inlineStr">
@@ -3687,30 +3744,34 @@
       </c>
       <c r="D27" s="18" t="inlineStr">
         <is>
-          <t>性能</t>
+          <t>白板 · 终端窗口</t>
         </is>
       </c>
       <c r="E27" s="18" t="inlineStr">
         <is>
-          <t>三项完成标准没测量：30 个窗口平移不掉帧（B1）、Electron 里 6 个终端打字延迟（T2，只量到 tmux-host 层）、空闲时 CPU 接近 0（G4）</t>
+          <t>在真窗口里拉小成摘要卡、再恢复，画面会不会乱没验证</t>
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr">
         <is>
-          <t>写测量脚本</t>
+          <t>按 E09 走一遍</t>
         </is>
       </c>
       <c r="G27" s="18" t="inlineStr">
         <is>
-          <t>流畅是一开始的要求之一</t>
+          <t>摘要卡是放下更多窗口的办法</t>
         </is>
       </c>
       <c r="H27" s="18" t="inlineStr">
         <is>
-          <t>用组装好的应用加调试端口测</t>
-        </is>
-      </c>
-      <c r="I27" s="20" t="inlineStr"/>
+          <t>手动验收 E09</t>
+        </is>
+      </c>
+      <c r="I27" s="20" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
       <c r="J27" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -3721,7 +3782,7 @@
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>Q27</t>
+          <t>Q25</t>
         </is>
       </c>
       <c r="B28" s="24" t="inlineStr">
@@ -3736,32 +3797,32 @@
       </c>
       <c r="D28" s="18" t="inlineStr">
         <is>
-          <t>apps/desktop · store</t>
+          <t>源代码管理面板</t>
         </is>
       </c>
       <c r="E28" s="18" t="inlineStr">
         <is>
-          <t>强杀应用进程（不是 ⌘Q）后再打开，布局和终端恢复没测过</t>
+          <t>单击被别的工作区占用的分支跳到那个框，没在真窗口里试</t>
         </is>
       </c>
       <c r="F28" s="18" t="inlineStr">
         <is>
-          <t>kill -9 主进程后再打开</t>
+          <t>按 E08 走一遍</t>
         </is>
       </c>
       <c r="G28" s="18" t="inlineStr">
         <is>
-          <t>崩溃后能不能恢复</t>
+          <t>辅助功能</t>
         </is>
       </c>
       <c r="H28" s="18" t="inlineStr">
         <is>
-          <t>手动试一次，再写进端到端</t>
+          <t>手动验收 E08</t>
         </is>
       </c>
       <c r="I28" s="20" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="J28" s="21" t="inlineStr">
@@ -3774,7 +3835,7 @@
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>Q28</t>
+          <t>Q26</t>
         </is>
       </c>
       <c r="B29" s="24" t="inlineStr">
@@ -3784,32 +3845,32 @@
       </c>
       <c r="C29" s="20" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>未验证</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
         <is>
-          <t>apps/desktop</t>
+          <t>性能</t>
         </is>
       </c>
       <c r="E29" s="18" t="inlineStr">
         <is>
-          <t>IPC 层的“统一超时包装”没找到，只有错误码透传</t>
+          <t>三项完成标准没测量：30 个窗口平移不掉帧（B1）、Electron 里 6 个终端打字延迟（T2，只量到 tmux-host 层）、空闲时 CPU 接近 0（G4）</t>
         </is>
       </c>
       <c r="F29" s="18" t="inlineStr">
         <is>
-          <t>看 apps/desktop/src/main/ipc.ts</t>
+          <t>写测量脚本</t>
         </is>
       </c>
       <c r="G29" s="18" t="inlineStr">
         <is>
-          <t>某个服务卡住时界面会一直等</t>
+          <t>流畅是一开始的要求之一</t>
         </is>
       </c>
       <c r="H29" s="18" t="inlineStr">
         <is>
-          <t>给 invoke 加默认超时</t>
+          <t>用组装好的应用加调试端口测</t>
         </is>
       </c>
       <c r="I29" s="20" t="inlineStr"/>
@@ -3823,7 +3884,7 @@
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
         <is>
-          <t>Q29</t>
+          <t>Q27</t>
         </is>
       </c>
       <c r="B30" s="24" t="inlineStr">
@@ -3838,30 +3899,34 @@
       </c>
       <c r="D30" s="18" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>apps/desktop · store</t>
         </is>
       </c>
       <c r="E30" s="18" t="inlineStr">
         <is>
-          <t>GitHub Actions 从没跑过；工作流里也没装 tmux，真 tmux 的测试在 CI 上会被跳过</t>
+          <t>强杀应用进程（不是 ⌘Q）后再打开，布局和终端恢复没测过</t>
         </is>
       </c>
       <c r="F30" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>kill -9 主进程后再打开</t>
         </is>
       </c>
       <c r="G30" s="18" t="inlineStr">
         <is>
-          <t>只能靠本机跑 pnpm check</t>
+          <t>崩溃后能不能恢复</t>
         </is>
       </c>
       <c r="H30" s="18" t="inlineStr">
         <is>
-          <t>给出仓库名后推送；工作流里 brew/apt 装 tmux 3.5+</t>
-        </is>
-      </c>
-      <c r="I30" s="20" t="inlineStr"/>
+          <t>手动试一次，再写进端到端</t>
+        </is>
+      </c>
+      <c r="I30" s="20" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J30" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -3872,7 +3937,7 @@
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
         <is>
-          <t>Q36</t>
+          <t>Q28</t>
         </is>
       </c>
       <c r="B31" s="24" t="inlineStr">
@@ -3887,34 +3952,30 @@
       </c>
       <c r="D31" s="18" t="inlineStr">
         <is>
-          <t>整体</t>
+          <t>apps/desktop</t>
         </is>
       </c>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>重启电脑后恢复会话（验收场景 14）还没做</t>
+          <t>IPC 层的“统一超时包装”没找到，只有错误码透传</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>看 apps/desktop/src/main/ipc.ts</t>
         </is>
       </c>
       <c r="G31" s="18" t="inlineStr">
         <is>
-          <t>属于 MVP 完整版</t>
+          <t>某个服务卡住时界面会一直等</t>
         </is>
       </c>
       <c r="H31" s="18" t="inlineStr">
         <is>
-          <t>按计划在 M4 做</t>
-        </is>
-      </c>
-      <c r="I31" s="20" t="inlineStr">
-        <is>
-          <t>E14</t>
-        </is>
-      </c>
+          <t>给 invoke 加默认超时</t>
+        </is>
+      </c>
+      <c r="I31" s="20" t="inlineStr"/>
       <c r="J31" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -3925,7 +3986,7 @@
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>Q37</t>
+          <t>Q29</t>
         </is>
       </c>
       <c r="B32" s="24" t="inlineStr">
@@ -3935,17 +3996,17 @@
       </c>
       <c r="C32" s="20" t="inlineStr">
         <is>
-          <t>缺失</t>
+          <t>未验证</t>
         </is>
       </c>
       <c r="D32" s="18" t="inlineStr">
         <is>
-          <t>apps/desktop</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="E32" s="18" t="inlineStr">
         <is>
-          <t>没有打包流程：better-sqlite3 的 asarUnpack、node-pty spawn-helper 权限、tmux.conf 和 agentdeck-notify 的资源路径都还没进打包配置</t>
+          <t>GitHub Actions 从没跑过；工作流里也没装 tmux，真 tmux 的测试在 CI 上会被跳过</t>
         </is>
       </c>
       <c r="F32" s="18" t="inlineStr">
@@ -3955,19 +4016,15 @@
       </c>
       <c r="G32" s="18" t="inlineStr">
         <is>
-          <t>现在只能从源码 pnpm dev 启动，不能放进程序坞</t>
+          <t>只能靠本机跑 pnpm check</t>
         </is>
       </c>
       <c r="H32" s="18" t="inlineStr">
         <is>
-          <t>加 electron-builder 配置，产出 .app</t>
-        </is>
-      </c>
-      <c r="I32" s="20" t="inlineStr">
-        <is>
-          <t>E20</t>
-        </is>
-      </c>
+          <t>给出仓库名后推送；工作流里 brew/apt 装 tmux 3.5+</t>
+        </is>
+      </c>
+      <c r="I32" s="20" t="inlineStr"/>
       <c r="J32" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -3978,12 +4035,12 @@
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>Q30</t>
-        </is>
-      </c>
-      <c r="B33" s="29" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Q31</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="C33" s="20" t="inlineStr">
@@ -3993,27 +4050,27 @@
       </c>
       <c r="D33" s="18" t="inlineStr">
         <is>
-          <t>白板</t>
+          <t>git</t>
         </is>
       </c>
       <c r="E33" s="18" t="inlineStr">
         <is>
-          <t>右下角有 React Flow 的水印</t>
+          <t>开发期间留下十几个已合并的分支和 worktree，面板 Repository 区和分支下拉里全列出来了（Q38 就是点到了其中一个）</t>
         </is>
       </c>
       <c r="F33" s="18" t="inlineStr">
         <is>
-          <t>看截图右下角</t>
+          <t>git worktree list</t>
         </is>
       </c>
       <c r="G33" s="18" t="inlineStr">
         <is>
-          <t>外观</t>
+          <t>列表很乱</t>
         </is>
       </c>
       <c r="H33" s="18" t="inlineStr">
         <is>
-          <t>关掉水印</t>
+          <t>确认后删掉已合并的 claude/* 分支和对应 worktree</t>
         </is>
       </c>
       <c r="I33" s="20" t="inlineStr"/>
@@ -4027,45 +4084,49 @@
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>Q31</t>
-        </is>
-      </c>
-      <c r="B34" s="29" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Q36</t>
+        </is>
+      </c>
+      <c r="B34" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="C34" s="20" t="inlineStr">
         <is>
-          <t>清理</t>
+          <t>缺失</t>
         </is>
       </c>
       <c r="D34" s="18" t="inlineStr">
         <is>
-          <t>git</t>
+          <t>整体</t>
         </is>
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>开发期间留下十几个已合并的分支和 worktree，面板 Repository 区全列出来了</t>
+          <t>重启电脑后恢复会话（验收场景 14）还没做</t>
         </is>
       </c>
       <c r="F34" s="18" t="inlineStr">
         <is>
-          <t>git worktree list</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G34" s="18" t="inlineStr">
         <is>
-          <t>列表很乱</t>
+          <t>属于 MVP 完整版</t>
         </is>
       </c>
       <c r="H34" s="18" t="inlineStr">
         <is>
-          <t>确认后删掉已合并的 claude/* 分支和对应 worktree</t>
-        </is>
-      </c>
-      <c r="I34" s="20" t="inlineStr"/>
+          <t>按计划在 M4 做</t>
+        </is>
+      </c>
+      <c r="I34" s="20" t="inlineStr">
+        <is>
+          <t>E14</t>
+        </is>
+      </c>
       <c r="J34" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -4076,45 +4137,49 @@
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>Q32</t>
-        </is>
-      </c>
-      <c r="B35" s="29" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>Q37</t>
+        </is>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="C35" s="20" t="inlineStr">
         <is>
-          <t>清理</t>
+          <t>缺失</t>
         </is>
       </c>
       <c r="D35" s="18" t="inlineStr">
         <is>
-          <t>开发环境</t>
+          <t>apps/desktop</t>
         </is>
       </c>
       <c r="E35" s="18" t="inlineStr">
         <is>
-          <t>Electron 二进制要手动下载一次（pnpm 10 不跑依赖的 postinstall）</t>
+          <t>没有打包流程：better-sqlite3 的 asarUnpack、node-pty spawn-helper 权限、tmux.conf 和 agentdeck-notify 的资源路径都还没进打包配置</t>
         </is>
       </c>
       <c r="F35" s="18" t="inlineStr">
         <is>
-          <t>新克隆后 pnpm dev 报 Electron uninstall</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G35" s="18" t="inlineStr">
         <is>
-          <t>新环境第一次启动会失败</t>
+          <t>现在只能从源码 pnpm dev 启动，不能放进程序坞</t>
         </is>
       </c>
       <c r="H35" s="18" t="inlineStr">
         <is>
-          <t>在 pnpm 配置里允许 electron 的安装脚本，或在根目录加 setup 脚本</t>
-        </is>
-      </c>
-      <c r="I35" s="20" t="inlineStr"/>
+          <t>加 electron-builder 配置，产出 .app</t>
+        </is>
+      </c>
+      <c r="I35" s="20" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
       <c r="J35" s="21" t="inlineStr">
         <is>
           <t>待处理</t>
@@ -4125,7 +4190,7 @@
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
         <is>
-          <t>Q33</t>
+          <t>Q30</t>
         </is>
       </c>
       <c r="B36" s="29" t="inlineStr">
@@ -4140,27 +4205,27 @@
       </c>
       <c r="D36" s="18" t="inlineStr">
         <is>
-          <t>开发环境</t>
+          <t>白板</t>
         </is>
       </c>
       <c r="E36" s="18" t="inlineStr">
         <is>
-          <t>dev 的 tmux 实例里留着 4 个演示会话，其中 2 个来自组装用的 worktree</t>
+          <t>右下角有 React Flow 的水印</t>
         </is>
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
-          <t>tmux -L agentdeck-desktop-dev ls</t>
+          <t>看截图右下角</t>
         </is>
       </c>
       <c r="G36" s="18" t="inlineStr">
         <is>
-          <t>无害，占一点资源</t>
+          <t>外观</t>
         </is>
       </c>
       <c r="H36" s="18" t="inlineStr">
         <is>
-          <t>验收完后 tmux -L agentdeck-desktop-dev kill-server</t>
+          <t>关掉水印</t>
         </is>
       </c>
       <c r="I36" s="20" t="inlineStr"/>
@@ -4174,7 +4239,7 @@
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
         <is>
-          <t>Q34</t>
+          <t>Q32</t>
         </is>
       </c>
       <c r="B37" s="29" t="inlineStr">
@@ -4184,32 +4249,32 @@
       </c>
       <c r="C37" s="20" t="inlineStr">
         <is>
-          <t>技术债</t>
+          <t>清理</t>
         </is>
       </c>
       <c r="D37" s="18" t="inlineStr">
         <is>
-          <t>agent-adapters 测试</t>
+          <t>开发环境</t>
         </is>
       </c>
       <c r="E37" s="18" t="inlineStr">
         <is>
-          <t>真 agent 测试会自动回答 codex 的“信任这个文件夹”，往用户的 codex 配置里写记录</t>
+          <t>Electron 二进制要手动下载一次（pnpm 10 不跑依赖的 postinstall）</t>
         </is>
       </c>
       <c r="F37" s="18" t="inlineStr">
         <is>
-          <t>看 real-agents.test.ts</t>
+          <t>新克隆后 pnpm dev 报 Electron uninstall</t>
         </is>
       </c>
       <c r="G37" s="18" t="inlineStr">
         <is>
-          <t>跑测试会改用户配置</t>
+          <t>新环境第一次启动会失败</t>
         </is>
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>测试里用临时 CODEX_HOME 和 CLAUDE_CONFIG_DIR</t>
+          <t>在 pnpm 配置里允许 electron 的安装脚本，或在根目录加 setup 脚本</t>
         </is>
       </c>
       <c r="I37" s="20" t="inlineStr"/>
@@ -4220,15 +4285,113 @@
       </c>
       <c r="K37" s="22" t="n"/>
     </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>Q33</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C38" s="20" t="inlineStr">
+        <is>
+          <t>清理</t>
+        </is>
+      </c>
+      <c r="D38" s="18" t="inlineStr">
+        <is>
+          <t>开发环境</t>
+        </is>
+      </c>
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>dev 的 tmux 实例里留着 4 个演示会话，其中 2 个来自组装用的 worktree</t>
+        </is>
+      </c>
+      <c r="F38" s="18" t="inlineStr">
+        <is>
+          <t>tmux -L agentdeck-desktop-dev ls</t>
+        </is>
+      </c>
+      <c r="G38" s="18" t="inlineStr">
+        <is>
+          <t>无害，占一点资源</t>
+        </is>
+      </c>
+      <c r="H38" s="18" t="inlineStr">
+        <is>
+          <t>验收完后 tmux -L agentdeck-desktop-dev kill-server</t>
+        </is>
+      </c>
+      <c r="I38" s="20" t="inlineStr"/>
+      <c r="J38" s="21" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="K38" s="22" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>Q34</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C39" s="20" t="inlineStr">
+        <is>
+          <t>技术债</t>
+        </is>
+      </c>
+      <c r="D39" s="18" t="inlineStr">
+        <is>
+          <t>agent-adapters 测试</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="inlineStr">
+        <is>
+          <t>真 agent 测试会自动回答 codex 的“信任这个文件夹”，往用户的 codex 配置里写记录</t>
+        </is>
+      </c>
+      <c r="F39" s="18" t="inlineStr">
+        <is>
+          <t>看 real-agents.test.ts</t>
+        </is>
+      </c>
+      <c r="G39" s="18" t="inlineStr">
+        <is>
+          <t>跑测试会改用户配置</t>
+        </is>
+      </c>
+      <c r="H39" s="18" t="inlineStr">
+        <is>
+          <t>测试里用临时 CODEX_HOME 和 CLAUDE_CONFIG_DIR</t>
+        </is>
+      </c>
+      <c r="I39" s="20" t="inlineStr"/>
+      <c r="J39" s="21" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="K39" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K37"/>
-  <conditionalFormatting sqref="J2:J37">
+  <autoFilter ref="A1:K39"/>
+  <conditionalFormatting sqref="J2:J39">
     <cfRule type="expression" priority="1" dxfId="1">
       <formula>$J2="已解决"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="J2:J39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"待处理,处理中,已解决,不处理"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4294,15 +4457,15 @@
         </is>
       </c>
       <c r="B5" s="34">
-        <f>COUNTIF('端到端用例'!$C$2:$C$24,A5)</f>
+        <f>COUNTIF('端到端用例'!$C$2:$C$25,A5)</f>
         <v/>
       </c>
       <c r="C5" s="34">
-        <f>COUNTIFS('端到端用例'!$C$2:$C$24,A5,'端到端用例'!$K$2:$K$24,"通过")</f>
+        <f>COUNTIFS('端到端用例'!$C$2:$C$25,A5,'端到端用例'!$K$2:$K$25,"通过")</f>
         <v/>
       </c>
       <c r="D5" s="34">
-        <f>COUNTIFS('端到端用例'!$C$2:$C$24,A5,'端到端用例'!$K$2:$K$24,"不通过")</f>
+        <f>COUNTIFS('端到端用例'!$C$2:$C$25,A5,'端到端用例'!$K$2:$K$25,"不通过")</f>
         <v/>
       </c>
     </row>
@@ -4313,15 +4476,15 @@
         </is>
       </c>
       <c r="B6" s="34">
-        <f>COUNTIF('端到端用例'!$C$2:$C$24,A6)</f>
+        <f>COUNTIF('端到端用例'!$C$2:$C$25,A6)</f>
         <v/>
       </c>
       <c r="C6" s="34">
-        <f>COUNTIFS('端到端用例'!$C$2:$C$24,A6,'端到端用例'!$K$2:$K$24,"通过")</f>
+        <f>COUNTIFS('端到端用例'!$C$2:$C$25,A6,'端到端用例'!$K$2:$K$25,"通过")</f>
         <v/>
       </c>
       <c r="D6" s="34">
-        <f>COUNTIFS('端到端用例'!$C$2:$C$24,A6,'端到端用例'!$K$2:$K$24,"不通过")</f>
+        <f>COUNTIFS('端到端用例'!$C$2:$C$25,A6,'端到端用例'!$K$2:$K$25,"不通过")</f>
         <v/>
       </c>
     </row>
@@ -4332,15 +4495,15 @@
         </is>
       </c>
       <c r="B7" s="34">
-        <f>COUNTIF('端到端用例'!$C$2:$C$24,A7)</f>
+        <f>COUNTIF('端到端用例'!$C$2:$C$25,A7)</f>
         <v/>
       </c>
       <c r="C7" s="34">
-        <f>COUNTIFS('端到端用例'!$C$2:$C$24,A7,'端到端用例'!$K$2:$K$24,"通过")</f>
+        <f>COUNTIFS('端到端用例'!$C$2:$C$25,A7,'端到端用例'!$K$2:$K$25,"通过")</f>
         <v/>
       </c>
       <c r="D7" s="34">
-        <f>COUNTIFS('端到端用例'!$C$2:$C$24,A7,'端到端用例'!$K$2:$K$24,"不通过")</f>
+        <f>COUNTIFS('端到端用例'!$C$2:$C$25,A7,'端到端用例'!$K$2:$K$25,"不通过")</f>
         <v/>
       </c>
     </row>
@@ -4351,15 +4514,15 @@
         </is>
       </c>
       <c r="B8" s="34">
-        <f>COUNTIF('端到端用例'!$C$2:$C$24,A8)</f>
+        <f>COUNTIF('端到端用例'!$C$2:$C$25,A8)</f>
         <v/>
       </c>
       <c r="C8" s="34">
-        <f>COUNTIFS('端到端用例'!$C$2:$C$24,A8,'端到端用例'!$K$2:$K$24,"通过")</f>
+        <f>COUNTIFS('端到端用例'!$C$2:$C$25,A8,'端到端用例'!$K$2:$K$25,"通过")</f>
         <v/>
       </c>
       <c r="D8" s="34">
-        <f>COUNTIFS('端到端用例'!$C$2:$C$24,A8,'端到端用例'!$K$2:$K$24,"不通过")</f>
+        <f>COUNTIFS('端到端用例'!$C$2:$C$25,A8,'端到端用例'!$K$2:$K$25,"不通过")</f>
         <v/>
       </c>
     </row>
@@ -4370,15 +4533,15 @@
         </is>
       </c>
       <c r="B9" s="34">
-        <f>COUNTIF('端到端用例'!$C$2:$C$24,A9)</f>
+        <f>COUNTIF('端到端用例'!$C$2:$C$25,A9)</f>
         <v/>
       </c>
       <c r="C9" s="34">
-        <f>COUNTIFS('端到端用例'!$C$2:$C$24,A9,'端到端用例'!$K$2:$K$24,"通过")</f>
+        <f>COUNTIFS('端到端用例'!$C$2:$C$25,A9,'端到端用例'!$K$2:$K$25,"通过")</f>
         <v/>
       </c>
       <c r="D9" s="34">
-        <f>COUNTIFS('端到端用例'!$C$2:$C$24,A9,'端到端用例'!$K$2:$K$24,"不通过")</f>
+        <f>COUNTIFS('端到端用例'!$C$2:$C$25,A9,'端到端用例'!$K$2:$K$25,"不通过")</f>
         <v/>
       </c>
     </row>
@@ -4430,11 +4593,11 @@
         </is>
       </c>
       <c r="B13" s="34">
-        <f>COUNTIF('问题清单'!$B$2:$B$37,A13)</f>
+        <f>COUNTIF('问题清单'!$B$2:$B$39,A13)</f>
         <v/>
       </c>
       <c r="C13" s="34">
-        <f>COUNTIFS('问题清单'!$B$2:$B$37,A13,'问题清单'!$J$2:$J$37,"已解决")</f>
+        <f>COUNTIFS('问题清单'!$B$2:$B$39,A13,'问题清单'!$J$2:$J$39,"已解决")</f>
         <v/>
       </c>
       <c r="D13" s="34">
@@ -4449,11 +4612,11 @@
         </is>
       </c>
       <c r="B14" s="34">
-        <f>COUNTIF('问题清单'!$B$2:$B$37,A14)</f>
+        <f>COUNTIF('问题清单'!$B$2:$B$39,A14)</f>
         <v/>
       </c>
       <c r="C14" s="34">
-        <f>COUNTIFS('问题清单'!$B$2:$B$37,A14,'问题清单'!$J$2:$J$37,"已解决")</f>
+        <f>COUNTIFS('问题清单'!$B$2:$B$39,A14,'问题清单'!$J$2:$J$39,"已解决")</f>
         <v/>
       </c>
       <c r="D14" s="34">
@@ -4468,11 +4631,11 @@
         </is>
       </c>
       <c r="B15" s="34">
-        <f>COUNTIF('问题清单'!$B$2:$B$37,A15)</f>
+        <f>COUNTIF('问题清单'!$B$2:$B$39,A15)</f>
         <v/>
       </c>
       <c r="C15" s="34">
-        <f>COUNTIFS('问题清单'!$B$2:$B$37,A15,'问题清单'!$J$2:$J$37,"已解决")</f>
+        <f>COUNTIFS('问题清单'!$B$2:$B$39,A15,'问题清单'!$J$2:$J$39,"已解决")</f>
         <v/>
       </c>
       <c r="D15" s="34">
@@ -4487,11 +4650,11 @@
         </is>
       </c>
       <c r="B16" s="34">
-        <f>COUNTIF('问题清单'!$B$2:$B$37,A16)</f>
+        <f>COUNTIF('问题清单'!$B$2:$B$39,A16)</f>
         <v/>
       </c>
       <c r="C16" s="34">
-        <f>COUNTIFS('问题清单'!$B$2:$B$37,A16,'问题清单'!$J$2:$J$37,"已解决")</f>
+        <f>COUNTIFS('问题清单'!$B$2:$B$39,A16,'问题清单'!$J$2:$J$39,"已解决")</f>
         <v/>
       </c>
       <c r="D16" s="34">
@@ -4547,11 +4710,11 @@
         </is>
       </c>
       <c r="B20" s="34">
-        <f>COUNTIF('端到端用例'!$B$2:$B$24,A20)</f>
+        <f>COUNTIF('端到端用例'!$B$2:$B$25,A20)</f>
         <v/>
       </c>
       <c r="C20" s="34">
-        <f>COUNTIFS('端到端用例'!$B$2:$B$24,A20,'端到端用例'!$K$2:$K$24,"通过")</f>
+        <f>COUNTIFS('端到端用例'!$B$2:$B$25,A20,'端到端用例'!$K$2:$K$25,"通过")</f>
         <v/>
       </c>
       <c r="D20" s="34">
@@ -4566,11 +4729,11 @@
         </is>
       </c>
       <c r="B21" s="34">
-        <f>COUNTIF('端到端用例'!$B$2:$B$24,A21)</f>
+        <f>COUNTIF('端到端用例'!$B$2:$B$25,A21)</f>
         <v/>
       </c>
       <c r="C21" s="34">
-        <f>COUNTIFS('端到端用例'!$B$2:$B$24,A21,'端到端用例'!$K$2:$K$24,"通过")</f>
+        <f>COUNTIFS('端到端用例'!$B$2:$B$25,A21,'端到端用例'!$K$2:$K$25,"通过")</f>
         <v/>
       </c>
       <c r="D21" s="34">
@@ -4585,11 +4748,11 @@
         </is>
       </c>
       <c r="B22" s="34">
-        <f>COUNTIF('端到端用例'!$B$2:$B$24,A22)</f>
+        <f>COUNTIF('端到端用例'!$B$2:$B$25,A22)</f>
         <v/>
       </c>
       <c r="C22" s="34">
-        <f>COUNTIFS('端到端用例'!$B$2:$B$24,A22,'端到端用例'!$K$2:$K$24,"通过")</f>
+        <f>COUNTIFS('端到端用例'!$B$2:$B$25,A22,'端到端用例'!$K$2:$K$25,"通过")</f>
         <v/>
       </c>
       <c r="D22" s="34">

</xml_diff>

<commit_message>
docs: mark Q38, Q39 fixed in the acceptance xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/status/AgentDeck-端到端用例与问题清单-2026-10-24.xlsx
+++ b/docs/status/AgentDeck-端到端用例与问题清单-2026-10-24.xlsx
@@ -221,10 +221,10 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -236,6 +236,9 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -243,9 +246,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -678,7 +678,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24，基于 main 01947e0（下午补了 E24、Q38、Q39）。证据来自各包测试、apps/desktop/ASSEMBLY_NOTES.md、2026-10-23 的组装和两次启动截图。</t>
+          <t>2026-10-24，基于 main 925c11f（下午补了 E24、Q38、Q39，Q38、Q39 已修）。证据来自各包测试、apps/desktop/ASSEMBLY_NOTES.md、2026-10-23 的组装和两次启动截图。</t>
         </is>
       </c>
     </row>
@@ -1007,42 +1007,42 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>⚠ 当前有问题</t>
-        </is>
-      </c>
-      <c r="D2" s="18" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>部分验证</t>
+        </is>
+      </c>
+      <c r="D2" s="19" t="inlineStr">
         <is>
           <t>在面板里给“主目录工作区”切换分支</t>
         </is>
       </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="E2" s="19" t="inlineStr">
         <is>
           <t>主目录工作区的框里开着终端（空闲也算）；项目是一个普通测试仓库，不要用 agenduck 本身</t>
         </is>
       </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="F2" s="19" t="inlineStr">
         <is>
           <t>1. 聚焦框里的终端
 2. 面板里单击分支按钮
 3. 单击另一个分支</t>
         </is>
       </c>
-      <c r="G2" s="18" t="inlineStr">
+      <c r="G2" s="19" t="inlineStr">
         <is>
           <t>UI：只要这个目录里有终端开着（不管 Running 还是 Idle），先弹确认，写明哪些终端在这个目录里、它们看到的文件会变；确认后才切换，框标题更新为新分支。
 后台：确认后才执行 git switch；切换后 workspace-service 更新记录并发 workspace.changed。</t>
         </is>
       </c>
-      <c r="H2" s="18" t="inlineStr">
+      <c r="H2" s="19" t="inlineStr">
         <is>
           <t>不会因为点错一下就把正在用的目录切到别的分支</t>
         </is>
       </c>
       <c r="I2" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 实际发生：在 agenduck 自己的主目录工作区里单击分支，没有任何确认就把仓库从 main 切到了一个遗留分支（终端都是 Idle，面板只在有改动或有 Running 的 agent 时才确认）；而 AgentDeck 正是从这个目录运行的，开发服务器立刻加载了旧代码，界面变成早期自检页并报错（Q38、Q39）</t>
+          <t>已修（925c11f）：只要目录里有终端开着就确认（Q38）；切 AgentDeck 自己运行的目录（agenduck）会被拒绝并提示（Q39）。在真窗口里用调试端口调用切分支已确认被拒绝；确认框请在一个测试仓库上点一遍验收。起因：2026-10-24 在 agenduck 的主目录工作区里单击分支，没确认就切到遗留分支，正在运行的 AgentDeck 热更新成旧代码</t>
         </is>
       </c>
       <c r="J2" s="20" t="inlineStr">
@@ -1069,35 +1069,35 @@
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D3" s="18" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>agent 停下来请求批准时，用户一眼看出是谁在等</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>框里有一个已信任文件夹的 claude；应用分别在前台、后台各试一次</t>
         </is>
       </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>1. 让 claude 执行一个需要批准的命令（例如 “run ls in a new shell”）
 2. 不点任何东西，观察 2 秒
 3. 切到别的应用，再触发一次</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr">
+      <c r="G3" s="19" t="inlineStr">
         <is>
           <t>UI：2 秒内窗口出现橙色边框，标题栏状态 Needs approval，框标题和顶栏显示 “1 waiting”，程序坞角标 1；应用在后台时弹系统通知 “claude in … needs approval”。
 后台：claude 的 PermissionRequest 钩子经 agentdeck-notify 送到钩子 socket，状态机进入 needs-approval 并广播 status.changed。</t>
         </is>
       </c>
-      <c r="H3" s="18" t="inlineStr">
+      <c r="H3" s="19" t="inlineStr">
         <is>
           <t>不用盯着每个终端，也知道哪个 agent 在等你</t>
         </is>
       </c>
-      <c r="I3" s="19" t="inlineStr">
+      <c r="I3" s="23" t="inlineStr">
         <is>
           <t>claude 还停在“信任这个文件夹”提示时，状态显示 Idle，不变橙（Q06）；真 claude 的批准请求从没端到端跑过（Q01）；系统通知没真弹过（Q14）</t>
         </is>
@@ -1126,35 +1126,35 @@
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>跳到在等你的窗口，直接批准，agent 继续干活</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>E04 的状态：有一个 claude 在 Needs approval</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="19" t="inlineStr">
         <is>
           <t>1. 按 ⌘J
 2. 在终端里按 claude 的“允许一次”键
 3. 观察状态</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="19" t="inlineStr">
         <is>
           <t>UI：白板平移到那个窗口并聚焦，橙色边框消失（状态点仍橙）；批准后状态变 Running，“1 waiting” 消失。
 后台：输入经 tmux-host 送进 claude；PostToolUse / 新输出让状态机回到 running。</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="H4" s="19" t="inlineStr">
         <is>
           <t>从发现到批准一气呵成，不用找窗口</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="I4" s="23" t="inlineStr">
         <is>
           <t>需求写的是“直接按 y”，但 claude 实测“允许一次”是 1 或回车（线 1 核对），y 不确定能用，需要定需求（Q12）；批准后回到运行中没测过（Q01）</t>
         </is>
@@ -1183,35 +1183,35 @@
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>同一个仓库开两个工作区，两个 claude 并行改代码互不影响</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>已有项目，已建好 feat/oauth 工作区（E02）</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>1. 再建一个 fix/rate-limit 工作区
 2. 两个框里各新开一个 claude，紧接着连续开
 3. 各让它改一个不同的文件</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="G5" s="19" t="inlineStr">
         <is>
           <t>UI：两个框各自显示自己的分支，两个 claude 都正常启动；右侧面板随聚焦切换，只显示各自 worktree 的改动。
 后台：两个 worktree 各有自己的 HEAD 和暂存区；两个 tmux 会话的工作目录分别是两个 worktree。</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>多个 agent 在同一仓库的不同分支上同时工作，改动不串</t>
         </is>
       </c>
-      <c r="I5" s="19" t="inlineStr">
+      <c r="I5" s="23" t="inlineStr">
         <is>
           <t>连着新建两个终端时，第二个可能误显示 “Previous session ended”（Q07）；两个真 claude 并行从没试过（Q03）</t>
         </is>
@@ -1240,34 +1240,34 @@
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>退出应用再打开，所有东西都还在</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>白板上有框和至少两个终端，其中一个在跑</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>1. ⌘Q 退出
 2. 再打开（pnpm dev）</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="G6" s="19" t="inlineStr">
         <is>
           <t>UI：框和窗口的位置、大小不变；终端接回，历史输出都在；状态和计时正确。
 后台：tmux 里的会话在应用退出期间一直在跑；重开时按保存的 terminalId 接回，状态机重新登记这些终端。</t>
         </is>
       </c>
-      <c r="H6" s="18" t="inlineStr">
+      <c r="H6" s="19" t="inlineStr">
         <is>
           <t>关应用不打断 agent 的工作</t>
         </is>
       </c>
-      <c r="I6" s="19" t="inlineStr">
+      <c r="I6" s="23" t="inlineStr">
         <is>
           <t>接回后状态都显示 “Idle · now”，开始时间没接上（Q08）；强杀进程（不是 ⌘Q）后恢复没测过（Q27）。位置和输出 2026-10-23 已验证</t>
         </is>
@@ -1296,35 +1296,35 @@
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>基于 main 新建一个分支工作区，开箱即用</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>已添加项目（E01）；项目里有 .env；设置了初始化命令（例如 pnpm install）</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>1. 右键 › New workspace…
 2. 选 New worktree、New branch，名字 feat/oauth，from main
 3. Create</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
+      <c r="G7" s="19" t="inlineStr">
         <is>
           <t>UI：框出现在右键的位置，标题 “项目 · feat/oauth”；框里自动开一个 Shell 运行初始化命令；右侧面板显示 feat/oauth。
 后台：git worktree add 建好目录并新建分支；.env 被复制过去；失败时已建的 worktree 和分支回滚。</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="H7" s="19" t="inlineStr">
         <is>
           <t>一个新分支的独立工作目录准备好了，agent 可以直接进去干活</t>
         </is>
       </c>
-      <c r="I7" s="19" t="inlineStr">
+      <c r="I7" s="23" t="inlineStr">
         <is>
           <t>从界面新建 worktree 在真窗口里从没走过（Q02）；开发模式下 worktree 放在 .agentdeck-dev 里借用的假主目录下，路径和正式版不同（Q19）</t>
         </is>
@@ -1343,7 +1343,7 @@
           <t>E15</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1353,35 +1353,35 @@
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>修改项目设置：基础分支、复制的文件、初始化命令</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>已添加项目</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>1. 顶栏 Projects ▾ › Manage projects…（或 Settings › Projects）
 2. 改基础分支和初始化命令
 3. 新建一个工作区验证</t>
         </is>
       </c>
-      <c r="G8" s="18" t="inlineStr">
+      <c r="G8" s="19" t="inlineStr">
         <is>
           <t>UI：有项目设置页，能看到并修改名称、路径、基础分支、worktree 位置、复制的文件、初始化命令。
 后台：设置写进 store，新建工作区时生效。</t>
         </is>
       </c>
-      <c r="H8" s="18" t="inlineStr">
+      <c r="H8" s="19" t="inlineStr">
         <is>
           <t>每个项目按自己的习惯建工作区</t>
         </is>
       </c>
-      <c r="I8" s="19" t="inlineStr">
+      <c r="I8" s="23" t="inlineStr">
         <is>
           <t>没有 Settings 界面：点 Settings 只是用系统程序打开 settings.json，Settings › Projects 不存在（Q13）</t>
         </is>
@@ -1400,7 +1400,7 @@
           <t>E16</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1410,34 +1410,34 @@
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>刚打开应用，右侧面板给出有用的信息</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>白板上有一个工作区框，还没有聚焦任何窗口</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>1. 打开应用，不点任何东西
 2. 单击框里的一个终端</t>
         </is>
       </c>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="G9" s="19" t="inlineStr">
         <is>
           <t>UI：没聚焦时提示怎么开始（例如 “Select a window to see its changes”）；聚焦后显示那个工作区的 git 状态。
 后台：面板只在聚焦变化时刷新一次。</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr">
+      <c r="H9" s="19" t="inlineStr">
         <is>
           <t>面板不说让人困惑的话</t>
         </is>
       </c>
-      <c r="I9" s="19" t="inlineStr">
+      <c r="I9" s="23" t="inlineStr">
         <is>
           <t>没聚焦任何窗口时也显示 “This window isn’t in a workspace.”（Q22，见重开截图）</t>
         </is>
@@ -1456,7 +1456,7 @@
           <t>E17</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1466,33 +1466,33 @@
           <t>⚠ 当前有问题</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>右键新建终端，菜单只列出能用的 agent</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>本机装了 claude 和 codex</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="19" t="inlineStr">
         <is>
           <t>1. 在白板空白处右键 › New terminal ▸</t>
         </is>
       </c>
-      <c r="G10" s="18" t="inlineStr">
+      <c r="G10" s="19" t="inlineStr">
         <is>
           <t>UI：列出 Claude、Codex、Shell，用适配器的名字显示；没装的不出现；选中后在点击的位置开终端。
 后台：agents.list() 返回已安装的 agent。</t>
         </is>
       </c>
-      <c r="H10" s="18" t="inlineStr">
+      <c r="H10" s="19" t="inlineStr">
         <is>
           <t>菜单里每一项都能用</t>
         </is>
       </c>
-      <c r="I10" s="19" t="inlineStr">
+      <c r="I10" s="23" t="inlineStr">
         <is>
           <t>白板按 agent id 而不是名字显示，并且会列出用不了的 custom；应用里先把 custom 藏掉了，白板包本身没改（Q21）</t>
         </is>
@@ -1516,39 +1516,39 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="C11" s="25" t="inlineStr">
+      <c r="C11" s="26" t="inlineStr">
         <is>
           <t>未验证</t>
         </is>
       </c>
-      <c r="D11" s="18" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>第一次打开应用，添加一个项目</t>
         </is>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>干净的数据目录（删掉 .agentdeck-dev 或设 AGENTDECK_DATA_DIR 到新目录）；有一个本地 git 仓库</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>1. 在白板空白处右键 › Add project…
 2. 在系统的选文件夹窗口里选仓库（试一次选它的子文件夹）</t>
         </is>
       </c>
-      <c r="G11" s="18" t="inlineStr">
+      <c r="G11" s="19" t="inlineStr">
         <is>
           <t>UI：系统选文件夹窗口出现；选完直接进入 New workspace 对话框，项目已选好；选子文件夹时提示用了仓库根目录。
 后台：projects 表多一条；基础分支自动识别为远端默认分支或 main。</t>
         </is>
       </c>
-      <c r="H11" s="18" t="inlineStr">
+      <c r="H11" s="19" t="inlineStr">
         <is>
           <t>加项目一步到位，直接进入建工作区</t>
         </is>
       </c>
-      <c r="I11" s="18" t="inlineStr">
+      <c r="I11" s="19" t="inlineStr">
         <is>
           <t>流程有单测；组装时用的是演示模式自动加项目，真窗口里没点过</t>
         </is>
@@ -1567,45 +1567,45 @@
           <t>E06</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C12" s="26" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>在框里跑 dev server，点链接就在白板上看效果</t>
         </is>
       </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
         <is>
           <t>框里有一个 Shell 终端；项目能跑 pnpm dev（或用 python3 -m http.server 8765 代替）</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F12" s="19" t="inlineStr">
         <is>
           <t>1. 在终端里运行 dev server
 2. 单击输出里的 localhost 地址
 3. 再单击一次同一个地址</t>
         </is>
       </c>
-      <c r="G12" s="18" t="inlineStr">
+      <c r="G12" s="19" t="inlineStr">
         <is>
           <t>UI：网页窗口出现在终端右边、同一个框里，页面正常显示；第二次单击聚焦并刷新已开的窗口，不新开。
 后台：port-watch 从输出里识别出地址；主进程把这个来源加入响应头改写名单。</t>
         </is>
       </c>
-      <c r="H12" s="18" t="inlineStr">
+      <c r="H12" s="19" t="inlineStr">
         <is>
           <t>写代码和看效果在同一个框里</t>
         </is>
       </c>
-      <c r="I12" s="18" t="inlineStr">
+      <c r="I12" s="19" t="inlineStr">
         <is>
           <t>组装时用 python http.server 点开过网页窗口；真 pnpm dev 和“第二次点击复用”没在真窗口里试</t>
         </is>
@@ -1625,40 +1625,40 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D13" s="18" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>在右侧面板里提交 agent 改的代码</t>
         </is>
       </c>
-      <c r="E13" s="18" t="inlineStr">
+      <c r="E13" s="19" t="inlineStr">
         <is>
           <t>某个工作区里有几个改动的文件；用一个测试分支，不要在 main 上提交</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="F13" s="19" t="inlineStr">
         <is>
           <t>1. 聚焦那个工作区里的终端
 2. 悬停文件单击 + 暂存两个
 3. 写提交信息，按 ⌘↩</t>
         </is>
       </c>
-      <c r="G13" s="18" t="inlineStr">
+      <c r="G13" s="19" t="inlineStr">
         <is>
           <t>UI：面板显示这个分支的更改，按文件夹树形排列；暂存后进 Staged Changes；提交后列表清空一部分，提交记录顶部出现这一条。
 后台：git add / git commit 在这个 worktree 里执行；提交后面板再刷新一次 status。</t>
         </is>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="19" t="inlineStr">
         <is>
           <t>不离开白板完成提交</t>
         </is>
       </c>
-      <c r="I13" s="18" t="inlineStr">
+      <c r="I13" s="19" t="inlineStr">
         <is>
           <t>暂存和取消暂存在真窗口里试过；真的提交没做（为了不改 main）</t>
         </is>
@@ -1673,45 +1673,45 @@
           <t>E08</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C14" s="25" t="inlineStr">
+      <c r="C14" s="26" t="inlineStr">
         <is>
           <t>未验证</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>想切到已被别的工作区占用的分支时，直接跳过去</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E14" s="19" t="inlineStr">
         <is>
           <t>同一仓库有 feat/oauth 和 fix/rate-limit 两个工作区（E03）</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>1. 聚焦 feat/oauth 里的终端
 2. 面板里单击分支按钮
 3. 单击灰显的 fix/rate-limit</t>
         </is>
       </c>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="G14" s="19" t="inlineStr">
         <is>
           <t>UI：fix/rate-limit 灰显并写着 “in fix/rate-limit”；单击后白板平移到那个框并聚焦。
 后台：分支列表来自 git worktree list；不执行任何 git 操作。</t>
         </is>
       </c>
-      <c r="H14" s="18" t="inlineStr">
+      <c r="H14" s="19" t="inlineStr">
         <is>
           <t>不会因为分支被占用而切换失败</t>
         </is>
       </c>
-      <c r="I14" s="18" t="inlineStr">
+      <c r="I14" s="19" t="inlineStr">
         <is>
           <t>面板有单测；需要第二个 worktree，组装时没试</t>
         </is>
@@ -1730,44 +1730,44 @@
           <t>E09</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>把终端拉小成摘要卡，腾出地方</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E15" s="19" t="inlineStr">
         <is>
           <t>框里有两个在跑的终端</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F15" s="19" t="inlineStr">
         <is>
           <t>1. 把两个终端的右下角往里拉到很小
 2. 单击其中一个摘要卡</t>
         </is>
       </c>
-      <c r="G15" s="18" t="inlineStr">
+      <c r="G15" s="19" t="inlineStr">
         <is>
           <t>UI：小于 320×200 时变成摘要卡，显示最后 3 行和状态，在等你的仍是橙色；单击恢复到拉小之前的大小并聚焦，画面不乱。
 后台：摘要卡用 capture-pane 取最后几行，不 attach；恢复时重新 attach。</t>
         </is>
       </c>
-      <c r="H15" s="18" t="inlineStr">
+      <c r="H15" s="19" t="inlineStr">
         <is>
           <t>一屏放下更多 agent，又不丢信息</t>
         </is>
       </c>
-      <c r="I15" s="18" t="inlineStr">
+      <c r="I15" s="19" t="inlineStr">
         <is>
           <t>白板和终端窗口都有单测；真窗口里没拉过</t>
         </is>
@@ -1786,44 +1786,44 @@
           <t>E11</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C16" s="25" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>未验证</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>在系统终端里接上同一个 agent 会话</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="19" t="inlineStr">
         <is>
           <t>有一个在跑的 claude 终端</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>1. 标题栏右键 › Open in system terminal
 2. 在两边各输入几个字</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="G16" s="19" t="inlineStr">
         <is>
           <t>UI：系统终端打开并显示同一个会话；两边的输入和输出同步。
 后台：执行 tmux -L agentdeck attach-session -t &lt;id&gt;。</t>
         </is>
       </c>
-      <c r="H16" s="18" t="inlineStr">
+      <c r="H16" s="19" t="inlineStr">
         <is>
           <t>需要时可以用自己习惯的终端接着干</t>
         </is>
       </c>
-      <c r="I16" s="18" t="inlineStr">
+      <c r="I16" s="19" t="inlineStr">
         <is>
           <t>命令拼装有单测；组装时没真点（会打开别的应用）</t>
         </is>
@@ -1842,45 +1842,45 @@
           <t>E12</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C17" s="26" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D17" s="18" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>删除工作区，连目录一起删</t>
         </is>
       </c>
-      <c r="E17" s="18" t="inlineStr">
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>一个 worktree 工作区，里面有一个未提交的改动；用测试分支</t>
         </is>
       </c>
-      <c r="F17" s="18" t="inlineStr">
+      <c r="F17" s="19" t="inlineStr">
         <is>
           <t>1. 右键框 › Delete workspace…
 2. 选 Also delete the worktree folder
 3. 确认；看到“有未提交的更改”再确认一次</t>
         </is>
       </c>
-      <c r="G17" s="18" t="inlineStr">
+      <c r="G17" s="19" t="inlineStr">
         <is>
           <t>UI：第一次确认后提示有未提交的更改，必须再确认；完成后框从白板消失。
 后台：git worktree remove --force；目录从磁盘消失，分支保留。</t>
         </is>
       </c>
-      <c r="H17" s="18" t="inlineStr">
+      <c r="H17" s="19" t="inlineStr">
         <is>
           <t>清理干净，又不会误删还没提交的工作</t>
         </is>
       </c>
-      <c r="I17" s="18" t="inlineStr">
+      <c r="I17" s="19" t="inlineStr">
         <is>
           <t>服务层有真 git 测试；真窗口里没走过。会删目录，要在测试仓库上试</t>
         </is>
@@ -1899,45 +1899,45 @@
           <t>E13</t>
         </is>
       </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C18" s="26" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>关掉窗口，agent 在后台继续，需要时通知你</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
         <is>
           <t>有一个在跑的 claude</t>
         </is>
       </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="F18" s="19" t="inlineStr">
         <is>
           <t>1. 单击窗口的关闭按钮（不是 ⌘Q）
 2. 等 claude 请求批准
 3. 单击系统通知</t>
         </is>
       </c>
-      <c r="G18" s="18" t="inlineStr">
+      <c r="G18" s="19" t="inlineStr">
         <is>
           <t>UI：窗口消失，应用留在程序坞；有批准请求时弹系统通知、角标变 1；单击通知窗口回来并跳到那个终端。
 后台：界面销毁但主进程和 tmux 连接还在；钩子照常到达。</t>
         </is>
       </c>
-      <c r="H18" s="18" t="inlineStr">
+      <c r="H18" s="19" t="inlineStr">
         <is>
           <t>关窗口不等于停工</t>
         </is>
       </c>
-      <c r="I18" s="18" t="inlineStr">
+      <c r="I18" s="19" t="inlineStr">
         <is>
           <t>关窗口后台继续、点程序坞图标回来在真窗口里试过；点系统通知没试</t>
         </is>
@@ -1956,45 +1956,45 @@
           <t>E18</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>部分验证</t>
         </is>
       </c>
-      <c r="D19" s="18" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>焦点在网页窗口里时，应用快捷键照样能用</t>
         </is>
       </c>
-      <c r="E19" s="18" t="inlineStr">
+      <c r="E19" s="19" t="inlineStr">
         <is>
           <t>白板上有一个网页窗口和一个终端</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="F19" s="19" t="inlineStr">
         <is>
           <t>1. 单击网页内容
 2. 用真键盘按 ⌘J、⌘B、⌘W、⌘0、⌘1
 3. 在网页里按 ⌘R</t>
         </is>
       </c>
-      <c r="G19" s="18" t="inlineStr">
+      <c r="G19" s="19" t="inlineStr">
         <is>
           <t>UI：⌘J / ⌘B / ⌘W / ⌘0 / ⌘1 照常生效；⌘R 只刷新这个网页，不重载整个应用。
 后台：快捷键注册成应用菜单的 accelerator。</t>
         </is>
       </c>
-      <c r="H19" s="18" t="inlineStr">
+      <c r="H19" s="19" t="inlineStr">
         <is>
           <t>不管焦点在哪，快捷键行为一致</t>
         </is>
       </c>
-      <c r="I19" s="18" t="inlineStr">
+      <c r="I19" s="19" t="inlineStr">
         <is>
           <t>只用菜单项触发过 ⌘B、⌘W；真键盘没试</t>
         </is>
@@ -2013,44 +2013,44 @@
           <t>E19</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C20" s="25" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
         <is>
           <t>未验证</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>没装 tmux 或版本太低时给出明确的指引</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>临时把 PATH 里的 tmux 去掉，或用一个低于 3.5 的 tmux</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>1. 启动应用
 2. 按提示安装后点 Retry</t>
         </is>
       </c>
-      <c r="G20" s="18" t="inlineStr">
+      <c r="G20" s="19" t="inlineStr">
         <is>
           <t>UI：显示说明页，写明需要 tmux ≥ 3.5 和 brew install tmux，有 Retry；装好后 Retry 能起来。
 后台：启动时检查 tmux -V；低于 3.5 抛 tmux-unavailable。</t>
         </is>
       </c>
-      <c r="H20" s="18" t="inlineStr">
+      <c r="H20" s="19" t="inlineStr">
         <is>
           <t>第一次用的人知道该做什么</t>
         </is>
       </c>
-      <c r="I20" s="18" t="inlineStr">
+      <c r="I20" s="19" t="inlineStr">
         <is>
           <t>版本检查有单测；说明页在真窗口里没看过</t>
         </is>
@@ -2065,44 +2065,44 @@
           <t>E20</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C21" s="25" t="inlineStr">
+      <c r="C21" s="26" t="inlineStr">
         <is>
           <t>未验证</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>从程序坞打开应用，agent 照样能联网、能登录</t>
         </is>
       </c>
-      <c r="E21" s="18" t="inlineStr">
+      <c r="E21" s="19" t="inlineStr">
         <is>
           <t>需要打包好的应用（现在还没有打包流程）</t>
         </is>
       </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="F21" s="19" t="inlineStr">
         <is>
           <t>1. 从程序坞或访达打开 AgentDeck
 2. 新开一个 claude，发一句话</t>
         </is>
       </c>
-      <c r="G21" s="18" t="inlineStr">
+      <c r="G21" s="19" t="inlineStr">
         <is>
           <t>UI：claude 正常回答，不出现 403 或找不到命令。
 后台：启动时读登录 shell 的环境（PATH、代理变量），传给 tmux-host 和适配器。</t>
         </is>
       </c>
-      <c r="H21" s="18" t="inlineStr">
+      <c r="H21" s="19" t="inlineStr">
         <is>
           <t>不管从哪里打开，体验都和终端里一样</t>
         </is>
       </c>
-      <c r="I21" s="18" t="inlineStr">
+      <c r="I21" s="19" t="inlineStr">
         <is>
           <t>只从终端里 pnpm dev 启动过，那时环境本来就是全的；从程序坞启动要等有打包版本（Q11、Q37）</t>
         </is>
@@ -2131,34 +2131,34 @@
           <t>已验证</t>
         </is>
       </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>右键在白板上开一个终端并使用</t>
         </is>
       </c>
-      <c r="E22" s="18" t="inlineStr">
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>应用已打开</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
+      <c r="F22" s="19" t="inlineStr">
         <is>
           <t>1. 空白处右键 › New terminal ▸ Shell
 2. 输入 git status</t>
         </is>
       </c>
-      <c r="G22" s="18" t="inlineStr">
+      <c r="G22" s="19" t="inlineStr">
         <is>
           <t>UI：在点击的位置出现终端，散放的终端在 ~ 运行；输出正常显示，状态 Running 后变 Idle。
 后台：tmux 里新建会话，窗格带 AGENTDECK_TERM；输出经 MessagePort 直达界面。</t>
         </is>
       </c>
-      <c r="H22" s="18" t="inlineStr">
+      <c r="H22" s="19" t="inlineStr">
         <is>
           <t>白板上直接用真终端</t>
         </is>
       </c>
-      <c r="I22" s="18" t="inlineStr">
+      <c r="I22" s="19" t="inlineStr">
         <is>
           <t>2026-10-23 组装时验证</t>
         </is>
@@ -2173,7 +2173,7 @@
           <t>E22</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B23" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2183,34 +2183,34 @@
           <t>已验证</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>关闭运行中的终端会结束进程</t>
         </is>
       </c>
-      <c r="E23" s="18" t="inlineStr">
+      <c r="E23" s="19" t="inlineStr">
         <is>
           <t>有一个在跑的终端</t>
         </is>
       </c>
-      <c r="F23" s="18" t="inlineStr">
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>1. 单击标题栏的关闭
 2. 在确认框里选结束并关闭</t>
         </is>
       </c>
-      <c r="G23" s="18" t="inlineStr">
+      <c r="G23" s="19" t="inlineStr">
         <is>
           <t>UI：先弹确认；确认后窗口消失。
 后台：tmux 会话被结束。</t>
         </is>
       </c>
-      <c r="H23" s="18" t="inlineStr">
+      <c r="H23" s="19" t="inlineStr">
         <is>
           <t>关窗口不会留下看不见的进程</t>
         </is>
       </c>
-      <c r="I23" s="18" t="inlineStr">
+      <c r="I23" s="19" t="inlineStr">
         <is>
           <t>2026-10-23 组装时验证</t>
         </is>
@@ -2225,7 +2225,7 @@
           <t>E23</t>
         </is>
       </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="B24" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2235,34 +2235,34 @@
           <t>已验证</t>
         </is>
       </c>
-      <c r="D24" s="18" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>在面板里暂存再取消暂存一个文件</t>
         </is>
       </c>
-      <c r="E24" s="18" t="inlineStr">
+      <c r="E24" s="19" t="inlineStr">
         <is>
           <t>工作区里有一个改动</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr">
+      <c r="F24" s="19" t="inlineStr">
         <is>
           <t>1. 单击文件旁的 +
 2. 再单击 −</t>
         </is>
       </c>
-      <c r="G24" s="18" t="inlineStr">
+      <c r="G24" s="19" t="inlineStr">
         <is>
           <t>UI：文件在 Changes 和 Staged Changes 之间移动。
 后台：git add / git restore --staged；git status 和界面一致。</t>
         </is>
       </c>
-      <c r="H24" s="18" t="inlineStr">
+      <c r="H24" s="19" t="inlineStr">
         <is>
           <t>暂存操作和命令行一致</t>
         </is>
       </c>
-      <c r="I24" s="18" t="inlineStr">
+      <c r="I24" s="19" t="inlineStr">
         <is>
           <t>2026-10-23 组装时验证（两次都对照了 git status）</t>
         </is>
@@ -2277,7 +2277,7 @@
           <t>E14</t>
         </is>
       </c>
-      <c r="B25" s="24" t="inlineStr">
+      <c r="B25" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -2287,34 +2287,34 @@
           <t>未实现</t>
         </is>
       </c>
-      <c r="D25" s="18" t="inlineStr">
+      <c r="D25" s="19" t="inlineStr">
         <is>
           <t>重启电脑后恢复上次的工作区和 agent 对话</t>
         </is>
       </c>
-      <c r="E25" s="18" t="inlineStr">
+      <c r="E25" s="19" t="inlineStr">
         <is>
           <t>电脑重启过（或 tmux kill-server 模拟）</t>
         </is>
       </c>
-      <c r="F25" s="18" t="inlineStr">
+      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>1. 打开应用
 2. 在 “Restore your last session?” 里选 Restore all</t>
         </is>
       </c>
-      <c r="G25" s="18" t="inlineStr">
+      <c r="G25" s="19" t="inlineStr">
         <is>
           <t>UI：弹出恢复提示；恢复后工作区和窗口在原位，claude 接回原来的对话，Shell 在原目录打开并填好命令。
 后台：按记录的会话 id 运行 claude --resume &lt;id&gt;、codex resume &lt;id&gt;。</t>
         </is>
       </c>
-      <c r="H25" s="18" t="inlineStr">
+      <c r="H25" s="19" t="inlineStr">
         <is>
           <t>重启不丢上下文</t>
         </is>
       </c>
-      <c r="I25" s="18" t="inlineStr">
+      <c r="I25" s="19" t="inlineStr">
         <is>
           <t>属于 MVP 完整版（M4 · X6），还没做</t>
         </is>
@@ -2441,27 +2441,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D2" s="18" t="inlineStr">
+      <c r="D2" s="19" t="inlineStr">
         <is>
           <t>agent-adapters · 整体</t>
         </is>
       </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="E2" s="19" t="inlineStr">
         <is>
           <t>真 claude 的完整一轮从没在应用里跑通：信任提示之后的 SessionStart → 输入 → PermissionRequest → 批准 → Stop</t>
         </is>
       </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="F2" s="19" t="inlineStr">
         <is>
           <t>在 claude 窗口选 Yes, I trust this folder，按 E04、E05 走一遍</t>
         </is>
       </c>
-      <c r="G2" s="18" t="inlineStr">
+      <c r="G2" s="19" t="inlineStr">
         <is>
           <t>“谁在等你”这个核心能力还没被真实验证</t>
         </is>
       </c>
-      <c r="H2" s="18" t="inlineStr">
+      <c r="H2" s="19" t="inlineStr">
         <is>
           <t>先手动验收 E04/E05；之后写进端到端测试</t>
         </is>
@@ -2494,27 +2494,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D3" s="18" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>workspace-service · 白板</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>从界面新建 worktree 工作区、在框里开终端，从没在真窗口里走过</t>
         </is>
       </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="F3" s="19" t="inlineStr">
         <is>
           <t>按 E01、E02 走一遍</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr">
+      <c r="G3" s="19" t="inlineStr">
         <is>
           <t>多分支并行的基础，没走过就不能说 MVP 可用</t>
         </is>
       </c>
-      <c r="H3" s="18" t="inlineStr">
+      <c r="H3" s="19" t="inlineStr">
         <is>
           <t>手动验收 E01/E02</t>
         </is>
@@ -2547,27 +2547,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>整体</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>同一仓库两个工作区、两个 claude 并行改代码，从没试过</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="19" t="inlineStr">
         <is>
           <t>按 E03 走一遍</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="19" t="inlineStr">
         <is>
           <t>这是产品的核心卖点</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="H4" s="19" t="inlineStr">
         <is>
           <t>手动验收 E03</t>
         </is>
@@ -2600,27 +2600,27 @@
           <t>缺失</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>e2e</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>没有端到端自动测试（任务 R2）：仓库里没有 Playwright、没有 e2e 目录；14 条验收场景都没自动化</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="G5" s="19" t="inlineStr">
         <is>
           <t>以后每次改动都要靠人工回归</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>用 Playwright 的 Electron 模式，先做能完全自动的 E01 E02 E06 E07 E09 E10 E12</t>
         </is>
@@ -2653,27 +2653,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>tmux-host · 终端窗口</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>F7 列的 9 项终端手感只能人看，都还没确认：颜色和框线字符、Esc / Shift+Enter / 多行粘贴、触控板滚动和回滚、拖选复制、和系统终端同时接上、claude 完成提醒等</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>照 packages/tmux-host/AGENTS.md「需要人工确认」逐项试</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="G6" s="19" t="inlineStr">
         <is>
           <t>终端是天天用的东西，手感不对很快就不想用</t>
         </is>
       </c>
-      <c r="H6" s="18" t="inlineStr">
+      <c r="H6" s="19" t="inlineStr">
         <is>
           <t>验收时逐项打勾，有问题记成新的 Q</t>
         </is>
@@ -2702,27 +2702,27 @@
           <t>缺陷</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>源代码管理面板 · 白板</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>在面板里单击分支会立刻切换，不确认：只有在有未提交改动或有 Running 的 agent 时才弹框；框里的终端是 Idle 时直接切。空闲的 agent 和 Shell 也在这个目录里，切分支会改掉它们眼前的文件</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>主目录工作区里开一个 Idle 的终端，在面板里单击另一个分支</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
+      <c r="G7" s="19" t="inlineStr">
         <is>
           <t>误点一下就切走正在用的目录；2026-10-24 验收时实际发生</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="H7" s="19" t="inlineStr">
         <is>
           <t>只要这个目录里有任何终端开着就先确认（白板把框里所有活着的终端传给面板，不只 Running 的）；确认框写清会受影响的终端</t>
         </is>
@@ -2734,10 +2734,14 @@
       </c>
       <c r="J7" s="21" t="inlineStr">
         <is>
-          <t>待处理</t>
-        </is>
-      </c>
-      <c r="K7" s="22" t="n"/>
+          <t>已解决</t>
+        </is>
+      </c>
+      <c r="K7" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-24 已修（925c11f）：只要目录里有终端开着就确认，确认框列出这些终端；面板加了测试</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -2755,27 +2759,27 @@
           <t>开发风险</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>apps/desktop · 开发流程</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>用 AgentDeck 管理 agenduck 仓库自己时，切换主目录的分支会改掉正在运行的 AgentDeck 的源代码，开发服务器热更新成旧代码，界面直接坏掉</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>在 agenduck 自己的主目录工作区里切到任何旧分支</t>
         </is>
       </c>
-      <c r="G8" s="18" t="inlineStr">
+      <c r="G8" s="19" t="inlineStr">
         <is>
           <t>验收和自举开发时很容易误伤；恢复要手动 git switch main 再重启</t>
         </is>
       </c>
-      <c r="H8" s="18" t="inlineStr">
+      <c r="H8" s="19" t="inlineStr">
         <is>
           <t>短期：验收用别的测试仓库，或在独立 worktree 里跑 pnpm dev；长期：应用检测到要切的目录就是自己运行的目录时拒绝并提示</t>
         </is>
@@ -2787,10 +2791,14 @@
       </c>
       <c r="J8" s="21" t="inlineStr">
         <is>
-          <t>待处理</t>
-        </is>
-      </c>
-      <c r="K8" s="22" t="n"/>
+          <t>已解决</t>
+        </is>
+      </c>
+      <c r="K8" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-24 已修（925c11f）：应用启动时找出自己运行的目录，界面对它切分支、建分支并切换、连目录删除都拒绝；真窗口里验证过</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -2798,7 +2806,7 @@
           <t>Q06</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2808,27 +2816,27 @@
           <t>缺陷</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>agent-adapters</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>claude 停在“信任这个文件夹”提示时，状态显示 Idle，应该算在等你</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>打开一个没信任过的目录里的 claude</t>
         </is>
       </c>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="G9" s="19" t="inlineStr">
         <is>
           <t>用户以为 claude 在空闲，其实它卡着等你</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr">
+      <c r="H9" s="19" t="inlineStr">
         <is>
           <t>状态机把启动后迟迟没有 SessionStart、且屏幕停住的情况算 needs-reply，或识别信任提示</t>
         </is>
@@ -2851,7 +2859,7 @@
           <t>Q07</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2861,27 +2869,27 @@
           <t>缺陷</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>终端窗口</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>连着新建两个终端时，第二个可能误显示 “Previous session ended”（它复用了 500 毫秒内的 terminals.list() 结果）</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="19" t="inlineStr">
         <is>
           <t>快速连开两个终端</t>
         </is>
       </c>
-      <c r="G10" s="18" t="inlineStr">
+      <c r="G10" s="19" t="inlineStr">
         <is>
           <t>用户以为终端没起来</t>
         </is>
       </c>
-      <c r="H10" s="18" t="inlineStr">
+      <c r="H10" s="19" t="inlineStr">
         <is>
           <t>新建后强制刷新列表，或按 terminalId 精确查询</t>
         </is>
@@ -2904,7 +2912,7 @@
           <t>Q09</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2914,27 +2922,27 @@
           <t>技术债</t>
         </is>
       </c>
-      <c r="D11" s="18" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>tmux-host</t>
         </is>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>pty.ts 自己声明了顶层 const require，和 electron-vite 注入的重名，终端进程一启动就崩；组装时在构建配置里绕过</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>去掉桌面构建配置里的绕过插件后启动</t>
         </is>
       </c>
-      <c r="G11" s="18" t="inlineStr">
+      <c r="G11" s="19" t="inlineStr">
         <is>
           <t>换构建工具或打包时会再炸</t>
         </is>
       </c>
-      <c r="H11" s="18" t="inlineStr">
+      <c r="H11" s="19" t="inlineStr">
         <is>
           <t>在 tmux-host 里改名，去掉绕过</t>
         </is>
@@ -2953,7 +2961,7 @@
           <t>Q10</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2963,27 +2971,27 @@
           <t>技术债</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>tmux-host</t>
         </is>
       </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
         <is>
           <t>打包后默认的 tmux.conf 路径不对，应用现在总是显式传路径</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F12" s="19" t="inlineStr">
         <is>
           <t>打包后不传路径启动</t>
         </is>
       </c>
-      <c r="G12" s="18" t="inlineStr">
+      <c r="G12" s="19" t="inlineStr">
         <is>
           <t>打包时容易漏</t>
         </is>
       </c>
-      <c r="H12" s="18" t="inlineStr">
+      <c r="H12" s="19" t="inlineStr">
         <is>
           <t>默认路径按打包后的资源目录算</t>
         </is>
@@ -3002,7 +3010,7 @@
           <t>Q11</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3012,27 +3020,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D13" s="18" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>apps/desktop</t>
         </is>
       </c>
-      <c r="E13" s="18" t="inlineStr">
+      <c r="E13" s="19" t="inlineStr">
         <is>
           <t>从程序坞打开时读登录 shell 环境（PATH、代理）没验证过：只从终端 pnpm dev 启动过，那时环境本来就全</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="F13" s="19" t="inlineStr">
         <is>
           <t>有打包版本后从程序坞打开，开 claude 发一句话</t>
         </is>
       </c>
-      <c r="G13" s="18" t="inlineStr">
+      <c r="G13" s="19" t="inlineStr">
         <is>
           <t>之前 403 就是缺代理变量导致的</t>
         </is>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="19" t="inlineStr">
         <is>
           <t>和 Q37 一起做</t>
         </is>
@@ -3055,7 +3063,7 @@
           <t>Q12</t>
         </is>
       </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3065,27 +3073,27 @@
           <t>需求不一致</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>需求 · agent-adapters</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E14" s="19" t="inlineStr">
         <is>
           <t>验收场景 5 写“直接按 y 批准”，claude 实测“允许一次”是 1 或回车，y 能不能用不确定</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>在 claude 的批准提示里按 y 试一次</t>
         </is>
       </c>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="G14" s="19" t="inlineStr">
         <is>
           <t>按错键可能选到别的选项</t>
         </is>
       </c>
-      <c r="H14" s="18" t="inlineStr">
+      <c r="H14" s="19" t="inlineStr">
         <is>
           <t>改需求写法为“按 agent 的允许一次键（claude 是 1）”，或实测 y 后定下</t>
         </is>
@@ -3108,7 +3116,7 @@
           <t>Q13</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3118,27 +3126,27 @@
           <t>缺失</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>白板 · apps/desktop</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E15" s="19" t="inlineStr">
         <is>
           <t>没有 Settings 界面：设置存在 settings.json，点 Settings 用系统程序打开它；需求里的 Settings › Projects、Settings › Agents 都没有</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F15" s="19" t="inlineStr">
         <is>
           <t>点顶栏 Settings</t>
         </is>
       </c>
-      <c r="G15" s="18" t="inlineStr">
+      <c r="G15" s="19" t="inlineStr">
         <is>
           <t>项目设置、agent 启动参数、破坏性命令名单都只能手改 JSON</t>
         </is>
       </c>
-      <c r="H15" s="18" t="inlineStr">
+      <c r="H15" s="19" t="inlineStr">
         <is>
           <t>先做 Projects 和 Agents 两页</t>
         </is>
@@ -3161,7 +3169,7 @@
           <t>Q14</t>
         </is>
       </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3171,27 +3179,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>apps/desktop</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="19" t="inlineStr">
         <is>
           <t>系统通知真弹出、单击后窗口回来并跳到终端，没验证</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>按 E13 走一遍</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="G16" s="19" t="inlineStr">
         <is>
           <t>后台提醒是“不用盯着”的关键</t>
         </is>
       </c>
-      <c r="H16" s="18" t="inlineStr">
+      <c r="H16" s="19" t="inlineStr">
         <is>
           <t>手动验收 E13</t>
         </is>
@@ -3214,7 +3222,7 @@
           <t>Q16</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3224,27 +3232,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D17" s="18" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>apps/desktop · 白板</t>
         </is>
       </c>
-      <c r="E17" s="18" t="inlineStr">
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>焦点在网页窗口里时，用真键盘按应用快捷键没验证过（只用菜单项触发过）</t>
         </is>
       </c>
-      <c r="F17" s="18" t="inlineStr">
+      <c r="F17" s="19" t="inlineStr">
         <is>
           <t>按 E18 走一遍</t>
         </is>
       </c>
-      <c r="G17" s="18" t="inlineStr">
+      <c r="G17" s="19" t="inlineStr">
         <is>
           <t>快捷键失灵会很烦</t>
         </is>
       </c>
-      <c r="H17" s="18" t="inlineStr">
+      <c r="H17" s="19" t="inlineStr">
         <is>
           <t>手动验收 E18</t>
         </is>
@@ -3267,7 +3275,7 @@
           <t>Q17</t>
         </is>
       </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3277,27 +3285,27 @@
           <t>技术债</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>contracts</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
         <is>
           <t>线 1 的 13 条接口意见没整理成 0.1.4：关闭确认不知道进程在不在跑、⌘K 只发 Ctrl+L 没清历史、拖入文件拿不到路径、没有打开外部链接、没有终端配色 token 等</t>
         </is>
       </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="F18" s="19" t="inlineStr">
         <is>
           <t>看 packages/tmux-host/CONTRACT_NOTES.md</t>
         </is>
       </c>
-      <c r="G18" s="18" t="inlineStr">
+      <c r="G18" s="19" t="inlineStr">
         <is>
           <t>这些地方现在是各包自己临时处理</t>
         </is>
       </c>
-      <c r="H18" s="18" t="inlineStr">
+      <c r="H18" s="19" t="inlineStr">
         <is>
           <t>出 contracts 0.1.4 并跟进实现</t>
         </is>
@@ -3316,7 +3324,7 @@
           <t>Q24</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3326,27 +3334,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D19" s="18" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>白板 · workspace-service</t>
         </is>
       </c>
-      <c r="E19" s="18" t="inlineStr">
+      <c r="E19" s="19" t="inlineStr">
         <is>
           <t>在真窗口里删除工作区并删目录没走过（会真删磁盘目录）</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="F19" s="19" t="inlineStr">
         <is>
           <t>在测试仓库上按 E12 走一遍</t>
         </is>
       </c>
-      <c r="G19" s="18" t="inlineStr">
+      <c r="G19" s="19" t="inlineStr">
         <is>
           <t>删除是不可逆操作，必须先验证</t>
         </is>
       </c>
-      <c r="H19" s="18" t="inlineStr">
+      <c r="H19" s="19" t="inlineStr">
         <is>
           <t>手动验收 E12</t>
         </is>
@@ -3369,7 +3377,7 @@
           <t>Q08</t>
         </is>
       </c>
-      <c r="B20" s="24" t="inlineStr">
+      <c r="B20" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3379,27 +3387,27 @@
           <t>缺陷</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>agent-adapters · contracts</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>重开应用后终端状态都显示 “Idle · now”，开始时间没接上</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>有终端在跑时 ⌘Q 再打开</t>
         </is>
       </c>
-      <c r="G20" s="18" t="inlineStr">
+      <c r="G20" s="19" t="inlineStr">
         <is>
           <t>计时不准，但不影响使用</t>
         </is>
       </c>
-      <c r="H20" s="18" t="inlineStr">
+      <c r="H20" s="19" t="inlineStr">
         <is>
           <t>状态机接受恢复时的真实开始时间</t>
         </is>
@@ -3422,7 +3430,7 @@
           <t>Q15</t>
         </is>
       </c>
-      <c r="B21" s="24" t="inlineStr">
+      <c r="B21" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3432,27 +3440,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>终端窗口 · apps/desktop</t>
         </is>
       </c>
-      <c r="E21" s="18" t="inlineStr">
+      <c r="E21" s="19" t="inlineStr">
         <is>
           <t>Open in system terminal 没真点过</t>
         </is>
       </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="F21" s="19" t="inlineStr">
         <is>
           <t>按 E11 走一遍</t>
         </is>
       </c>
-      <c r="G21" s="18" t="inlineStr">
+      <c r="G21" s="19" t="inlineStr">
         <is>
           <t>辅助功能</t>
         </is>
       </c>
-      <c r="H21" s="18" t="inlineStr">
+      <c r="H21" s="19" t="inlineStr">
         <is>
           <t>手动验收 E11</t>
         </is>
@@ -3475,7 +3483,7 @@
           <t>Q18</t>
         </is>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B22" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3485,27 +3493,27 @@
           <t>技术债</t>
         </is>
       </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>白板 · 网页窗口 · git · agent</t>
         </is>
       </c>
-      <c r="E22" s="18" t="inlineStr">
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>线 2–5 还没把 contracts 0.1.3 的新字段用进代码：白板仍按 type === "terminal" 写特例、reuseKey 不随白板保存、网页窗口用本地的 reloadToken、远端分支和接回已有 worktree 没实现等</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
+      <c r="F22" s="19" t="inlineStr">
         <is>
           <t>看各包 CONTRACT_NOTES.md 开头的“待跟进”</t>
         </is>
       </c>
-      <c r="G22" s="18" t="inlineStr">
+      <c r="G22" s="19" t="inlineStr">
         <is>
           <t>加新窗口类型时要改白板</t>
         </is>
       </c>
-      <c r="H22" s="18" t="inlineStr">
+      <c r="H22" s="19" t="inlineStr">
         <is>
           <t>各包跟进一轮</t>
         </is>
@@ -3524,7 +3532,7 @@
           <t>Q19</t>
         </is>
       </c>
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B23" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3534,27 +3542,27 @@
           <t>缺失</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>workspace-service</t>
         </is>
       </c>
-      <c r="E23" s="18" t="inlineStr">
+      <c r="E23" s="19" t="inlineStr">
         <is>
           <t>没有“worktree 放在哪”的选项，开发模式下借用 .agentdeck-dev 里的假主目录</t>
         </is>
       </c>
-      <c r="F23" s="18" t="inlineStr">
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>开发模式下新建 worktree，看它的路径</t>
         </is>
       </c>
-      <c r="G23" s="18" t="inlineStr">
+      <c r="G23" s="19" t="inlineStr">
         <is>
           <t>开发和正式版路径不一致</t>
         </is>
       </c>
-      <c r="H23" s="18" t="inlineStr">
+      <c r="H23" s="19" t="inlineStr">
         <is>
           <t>给 workspace-service 加 worktreeRoot 参数</t>
         </is>
@@ -3577,7 +3585,7 @@
           <t>Q20</t>
         </is>
       </c>
-      <c r="B24" s="24" t="inlineStr">
+      <c r="B24" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3587,27 +3595,27 @@
           <t>缺陷</t>
         </is>
       </c>
-      <c r="D24" s="18" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>白板</t>
         </is>
       </c>
-      <c r="E24" s="18" t="inlineStr">
+      <c r="E24" s="19" t="inlineStr">
         <is>
           <t>第二次调用 start() 在白板加载完之前就返回</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr">
+      <c r="F24" s="19" t="inlineStr">
         <is>
           <t>连续调用两次 controller.start()</t>
         </is>
       </c>
-      <c r="G24" s="18" t="inlineStr">
+      <c r="G24" s="19" t="inlineStr">
         <is>
           <t>应用里已绕过（先 start 再渲染）</t>
         </is>
       </c>
-      <c r="H24" s="18" t="inlineStr">
+      <c r="H24" s="19" t="inlineStr">
         <is>
           <t>让 start() 返回同一个 Promise</t>
         </is>
@@ -3626,7 +3634,7 @@
           <t>Q21</t>
         </is>
       </c>
-      <c r="B25" s="24" t="inlineStr">
+      <c r="B25" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3636,27 +3644,27 @@
           <t>缺陷</t>
         </is>
       </c>
-      <c r="D25" s="18" t="inlineStr">
+      <c r="D25" s="19" t="inlineStr">
         <is>
           <t>白板</t>
         </is>
       </c>
-      <c r="E25" s="18" t="inlineStr">
+      <c r="E25" s="19" t="inlineStr">
         <is>
           <t>新建终端菜单会列出用不了的 custom，并按 agent id 而不是名字显示</t>
         </is>
       </c>
-      <c r="F25" s="18" t="inlineStr">
+      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>右键 › New terminal ▸</t>
         </is>
       </c>
-      <c r="G25" s="18" t="inlineStr">
+      <c r="G25" s="19" t="inlineStr">
         <is>
           <t>应用里先藏了 custom</t>
         </is>
       </c>
-      <c r="H25" s="18" t="inlineStr">
+      <c r="H25" s="19" t="inlineStr">
         <is>
           <t>按 AgentInfo.label 显示，过滤 custom</t>
         </is>
@@ -3679,7 +3687,7 @@
           <t>Q22</t>
         </is>
       </c>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B26" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3689,27 +3697,27 @@
           <t>缺陷</t>
         </is>
       </c>
-      <c r="D26" s="18" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
         <is>
           <t>源代码管理面板</t>
         </is>
       </c>
-      <c r="E26" s="18" t="inlineStr">
+      <c r="E26" s="19" t="inlineStr">
         <is>
           <t>没有聚焦任何窗口时也显示 “This window isn’t in a workspace.”</t>
         </is>
       </c>
-      <c r="F26" s="18" t="inlineStr">
+      <c r="F26" s="19" t="inlineStr">
         <is>
           <t>打开应用不点任何东西</t>
         </is>
       </c>
-      <c r="G26" s="18" t="inlineStr">
+      <c r="G26" s="19" t="inlineStr">
         <is>
           <t>文案让人困惑</t>
         </is>
       </c>
-      <c r="H26" s="18" t="inlineStr">
+      <c r="H26" s="19" t="inlineStr">
         <is>
           <t>区分“没聚焦”和“聚焦的是散放窗口”</t>
         </is>
@@ -3732,7 +3740,7 @@
           <t>Q23</t>
         </is>
       </c>
-      <c r="B27" s="24" t="inlineStr">
+      <c r="B27" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3742,27 +3750,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D27" s="18" t="inlineStr">
+      <c r="D27" s="19" t="inlineStr">
         <is>
           <t>白板 · 终端窗口</t>
         </is>
       </c>
-      <c r="E27" s="18" t="inlineStr">
+      <c r="E27" s="19" t="inlineStr">
         <is>
           <t>在真窗口里拉小成摘要卡、再恢复，画面会不会乱没验证</t>
         </is>
       </c>
-      <c r="F27" s="18" t="inlineStr">
+      <c r="F27" s="19" t="inlineStr">
         <is>
           <t>按 E09 走一遍</t>
         </is>
       </c>
-      <c r="G27" s="18" t="inlineStr">
+      <c r="G27" s="19" t="inlineStr">
         <is>
           <t>摘要卡是放下更多窗口的办法</t>
         </is>
       </c>
-      <c r="H27" s="18" t="inlineStr">
+      <c r="H27" s="19" t="inlineStr">
         <is>
           <t>手动验收 E09</t>
         </is>
@@ -3785,7 +3793,7 @@
           <t>Q25</t>
         </is>
       </c>
-      <c r="B28" s="24" t="inlineStr">
+      <c r="B28" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3795,27 +3803,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D28" s="18" t="inlineStr">
+      <c r="D28" s="19" t="inlineStr">
         <is>
           <t>源代码管理面板</t>
         </is>
       </c>
-      <c r="E28" s="18" t="inlineStr">
+      <c r="E28" s="19" t="inlineStr">
         <is>
           <t>单击被别的工作区占用的分支跳到那个框，没在真窗口里试</t>
         </is>
       </c>
-      <c r="F28" s="18" t="inlineStr">
+      <c r="F28" s="19" t="inlineStr">
         <is>
           <t>按 E08 走一遍</t>
         </is>
       </c>
-      <c r="G28" s="18" t="inlineStr">
+      <c r="G28" s="19" t="inlineStr">
         <is>
           <t>辅助功能</t>
         </is>
       </c>
-      <c r="H28" s="18" t="inlineStr">
+      <c r="H28" s="19" t="inlineStr">
         <is>
           <t>手动验收 E08</t>
         </is>
@@ -3838,7 +3846,7 @@
           <t>Q26</t>
         </is>
       </c>
-      <c r="B29" s="24" t="inlineStr">
+      <c r="B29" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3848,27 +3856,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D29" s="18" t="inlineStr">
+      <c r="D29" s="19" t="inlineStr">
         <is>
           <t>性能</t>
         </is>
       </c>
-      <c r="E29" s="18" t="inlineStr">
+      <c r="E29" s="19" t="inlineStr">
         <is>
           <t>三项完成标准没测量：30 个窗口平移不掉帧（B1）、Electron 里 6 个终端打字延迟（T2，只量到 tmux-host 层）、空闲时 CPU 接近 0（G4）</t>
         </is>
       </c>
-      <c r="F29" s="18" t="inlineStr">
+      <c r="F29" s="19" t="inlineStr">
         <is>
           <t>写测量脚本</t>
         </is>
       </c>
-      <c r="G29" s="18" t="inlineStr">
+      <c r="G29" s="19" t="inlineStr">
         <is>
           <t>流畅是一开始的要求之一</t>
         </is>
       </c>
-      <c r="H29" s="18" t="inlineStr">
+      <c r="H29" s="19" t="inlineStr">
         <is>
           <t>用组装好的应用加调试端口测</t>
         </is>
@@ -3887,7 +3895,7 @@
           <t>Q27</t>
         </is>
       </c>
-      <c r="B30" s="24" t="inlineStr">
+      <c r="B30" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3897,27 +3905,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>apps/desktop · store</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
+      <c r="E30" s="19" t="inlineStr">
         <is>
           <t>强杀应用进程（不是 ⌘Q）后再打开，布局和终端恢复没测过</t>
         </is>
       </c>
-      <c r="F30" s="18" t="inlineStr">
+      <c r="F30" s="19" t="inlineStr">
         <is>
           <t>kill -9 主进程后再打开</t>
         </is>
       </c>
-      <c r="G30" s="18" t="inlineStr">
+      <c r="G30" s="19" t="inlineStr">
         <is>
           <t>崩溃后能不能恢复</t>
         </is>
       </c>
-      <c r="H30" s="18" t="inlineStr">
+      <c r="H30" s="19" t="inlineStr">
         <is>
           <t>手动试一次，再写进端到端</t>
         </is>
@@ -3940,7 +3948,7 @@
           <t>Q28</t>
         </is>
       </c>
-      <c r="B31" s="24" t="inlineStr">
+      <c r="B31" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3950,27 +3958,27 @@
           <t>缺失</t>
         </is>
       </c>
-      <c r="D31" s="18" t="inlineStr">
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>apps/desktop</t>
         </is>
       </c>
-      <c r="E31" s="18" t="inlineStr">
+      <c r="E31" s="19" t="inlineStr">
         <is>
           <t>IPC 层的“统一超时包装”没找到，只有错误码透传</t>
         </is>
       </c>
-      <c r="F31" s="18" t="inlineStr">
+      <c r="F31" s="19" t="inlineStr">
         <is>
           <t>看 apps/desktop/src/main/ipc.ts</t>
         </is>
       </c>
-      <c r="G31" s="18" t="inlineStr">
+      <c r="G31" s="19" t="inlineStr">
         <is>
           <t>某个服务卡住时界面会一直等</t>
         </is>
       </c>
-      <c r="H31" s="18" t="inlineStr">
+      <c r="H31" s="19" t="inlineStr">
         <is>
           <t>给 invoke 加默认超时</t>
         </is>
@@ -3989,7 +3997,7 @@
           <t>Q29</t>
         </is>
       </c>
-      <c r="B32" s="24" t="inlineStr">
+      <c r="B32" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3999,27 +4007,27 @@
           <t>未验证</t>
         </is>
       </c>
-      <c r="D32" s="18" t="inlineStr">
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>CI</t>
         </is>
       </c>
-      <c r="E32" s="18" t="inlineStr">
+      <c r="E32" s="19" t="inlineStr">
         <is>
           <t>GitHub Actions 从没跑过；工作流里也没装 tmux，真 tmux 的测试在 CI 上会被跳过</t>
         </is>
       </c>
-      <c r="F32" s="18" t="inlineStr">
+      <c r="F32" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G32" s="18" t="inlineStr">
+      <c r="G32" s="19" t="inlineStr">
         <is>
           <t>只能靠本机跑 pnpm check</t>
         </is>
       </c>
-      <c r="H32" s="18" t="inlineStr">
+      <c r="H32" s="19" t="inlineStr">
         <is>
           <t>给出仓库名后推送；工作流里 brew/apt 装 tmux 3.5+</t>
         </is>
@@ -4038,7 +4046,7 @@
           <t>Q31</t>
         </is>
       </c>
-      <c r="B33" s="24" t="inlineStr">
+      <c r="B33" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -4048,27 +4056,27 @@
           <t>清理</t>
         </is>
       </c>
-      <c r="D33" s="18" t="inlineStr">
+      <c r="D33" s="19" t="inlineStr">
         <is>
           <t>git</t>
         </is>
       </c>
-      <c r="E33" s="18" t="inlineStr">
+      <c r="E33" s="19" t="inlineStr">
         <is>
           <t>开发期间留下十几个已合并的分支和 worktree，面板 Repository 区和分支下拉里全列出来了（Q38 就是点到了其中一个）</t>
         </is>
       </c>
-      <c r="F33" s="18" t="inlineStr">
+      <c r="F33" s="19" t="inlineStr">
         <is>
           <t>git worktree list</t>
         </is>
       </c>
-      <c r="G33" s="18" t="inlineStr">
+      <c r="G33" s="19" t="inlineStr">
         <is>
           <t>列表很乱</t>
         </is>
       </c>
-      <c r="H33" s="18" t="inlineStr">
+      <c r="H33" s="19" t="inlineStr">
         <is>
           <t>确认后删掉已合并的 claude/* 分支和对应 worktree</t>
         </is>
@@ -4087,7 +4095,7 @@
           <t>Q36</t>
         </is>
       </c>
-      <c r="B34" s="24" t="inlineStr">
+      <c r="B34" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -4097,27 +4105,27 @@
           <t>缺失</t>
         </is>
       </c>
-      <c r="D34" s="18" t="inlineStr">
+      <c r="D34" s="19" t="inlineStr">
         <is>
           <t>整体</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
+      <c r="E34" s="19" t="inlineStr">
         <is>
           <t>重启电脑后恢复会话（验收场景 14）还没做</t>
         </is>
       </c>
-      <c r="F34" s="18" t="inlineStr">
+      <c r="F34" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G34" s="18" t="inlineStr">
+      <c r="G34" s="19" t="inlineStr">
         <is>
           <t>属于 MVP 完整版</t>
         </is>
       </c>
-      <c r="H34" s="18" t="inlineStr">
+      <c r="H34" s="19" t="inlineStr">
         <is>
           <t>按计划在 M4 做</t>
         </is>
@@ -4140,7 +4148,7 @@
           <t>Q37</t>
         </is>
       </c>
-      <c r="B35" s="24" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -4150,27 +4158,27 @@
           <t>缺失</t>
         </is>
       </c>
-      <c r="D35" s="18" t="inlineStr">
+      <c r="D35" s="19" t="inlineStr">
         <is>
           <t>apps/desktop</t>
         </is>
       </c>
-      <c r="E35" s="18" t="inlineStr">
+      <c r="E35" s="19" t="inlineStr">
         <is>
           <t>没有打包流程：better-sqlite3 的 asarUnpack、node-pty spawn-helper 权限、tmux.conf 和 agentdeck-notify 的资源路径都还没进打包配置</t>
         </is>
       </c>
-      <c r="F35" s="18" t="inlineStr">
+      <c r="F35" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G35" s="18" t="inlineStr">
+      <c r="G35" s="19" t="inlineStr">
         <is>
           <t>现在只能从源码 pnpm dev 启动，不能放进程序坞</t>
         </is>
       </c>
-      <c r="H35" s="18" t="inlineStr">
+      <c r="H35" s="19" t="inlineStr">
         <is>
           <t>加 electron-builder 配置，产出 .app</t>
         </is>
@@ -4203,27 +4211,27 @@
           <t>清理</t>
         </is>
       </c>
-      <c r="D36" s="18" t="inlineStr">
+      <c r="D36" s="19" t="inlineStr">
         <is>
           <t>白板</t>
         </is>
       </c>
-      <c r="E36" s="18" t="inlineStr">
+      <c r="E36" s="19" t="inlineStr">
         <is>
           <t>右下角有 React Flow 的水印</t>
         </is>
       </c>
-      <c r="F36" s="18" t="inlineStr">
+      <c r="F36" s="19" t="inlineStr">
         <is>
           <t>看截图右下角</t>
         </is>
       </c>
-      <c r="G36" s="18" t="inlineStr">
+      <c r="G36" s="19" t="inlineStr">
         <is>
           <t>外观</t>
         </is>
       </c>
-      <c r="H36" s="18" t="inlineStr">
+      <c r="H36" s="19" t="inlineStr">
         <is>
           <t>关掉水印</t>
         </is>
@@ -4252,27 +4260,27 @@
           <t>清理</t>
         </is>
       </c>
-      <c r="D37" s="18" t="inlineStr">
+      <c r="D37" s="19" t="inlineStr">
         <is>
           <t>开发环境</t>
         </is>
       </c>
-      <c r="E37" s="18" t="inlineStr">
+      <c r="E37" s="19" t="inlineStr">
         <is>
           <t>Electron 二进制要手动下载一次（pnpm 10 不跑依赖的 postinstall）</t>
         </is>
       </c>
-      <c r="F37" s="18" t="inlineStr">
+      <c r="F37" s="19" t="inlineStr">
         <is>
           <t>新克隆后 pnpm dev 报 Electron uninstall</t>
         </is>
       </c>
-      <c r="G37" s="18" t="inlineStr">
+      <c r="G37" s="19" t="inlineStr">
         <is>
           <t>新环境第一次启动会失败</t>
         </is>
       </c>
-      <c r="H37" s="18" t="inlineStr">
+      <c r="H37" s="19" t="inlineStr">
         <is>
           <t>在 pnpm 配置里允许 electron 的安装脚本，或在根目录加 setup 脚本</t>
         </is>
@@ -4301,27 +4309,27 @@
           <t>清理</t>
         </is>
       </c>
-      <c r="D38" s="18" t="inlineStr">
+      <c r="D38" s="19" t="inlineStr">
         <is>
           <t>开发环境</t>
         </is>
       </c>
-      <c r="E38" s="18" t="inlineStr">
+      <c r="E38" s="19" t="inlineStr">
         <is>
           <t>dev 的 tmux 实例里留着 4 个演示会话，其中 2 个来自组装用的 worktree</t>
         </is>
       </c>
-      <c r="F38" s="18" t="inlineStr">
+      <c r="F38" s="19" t="inlineStr">
         <is>
           <t>tmux -L agentdeck-desktop-dev ls</t>
         </is>
       </c>
-      <c r="G38" s="18" t="inlineStr">
+      <c r="G38" s="19" t="inlineStr">
         <is>
           <t>无害，占一点资源</t>
         </is>
       </c>
-      <c r="H38" s="18" t="inlineStr">
+      <c r="H38" s="19" t="inlineStr">
         <is>
           <t>验收完后 tmux -L agentdeck-desktop-dev kill-server</t>
         </is>
@@ -4350,27 +4358,27 @@
           <t>技术债</t>
         </is>
       </c>
-      <c r="D39" s="18" t="inlineStr">
+      <c r="D39" s="19" t="inlineStr">
         <is>
           <t>agent-adapters 测试</t>
         </is>
       </c>
-      <c r="E39" s="18" t="inlineStr">
+      <c r="E39" s="19" t="inlineStr">
         <is>
           <t>真 agent 测试会自动回答 codex 的“信任这个文件夹”，往用户的 codex 配置里写记录</t>
         </is>
       </c>
-      <c r="F39" s="18" t="inlineStr">
+      <c r="F39" s="19" t="inlineStr">
         <is>
           <t>看 real-agents.test.ts</t>
         </is>
       </c>
-      <c r="G39" s="18" t="inlineStr">
+      <c r="G39" s="19" t="inlineStr">
         <is>
           <t>跑测试会改用户配置</t>
         </is>
       </c>
-      <c r="H39" s="18" t="inlineStr">
+      <c r="H39" s="19" t="inlineStr">
         <is>
           <t>测试里用临时 CODEX_HOME 和 CLAUDE_CONFIG_DIR</t>
         </is>

</xml_diff>